<commit_message>
Add the data behind each figure to the Excel Figures tab
Each report figure now has its data table on the right, as live
formulas: key numbers, change vs the fish-only pond, global warming by
process, nitrogen fate, process shares (heatmap), KPI scorecard,
environmental profile, framework steps and margin to target.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LS2wYESwFTwwPUQtk712Bb
</commit_message>
<xml_diff>
--- a/excel/IMTA_KPI_decision_tool.xlsx
+++ b/excel/IMTA_KPI_decision_tool.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1107" uniqueCount="454">
   <si>
     <t xml:space="preserve">Pond IMTA vs fish polyculture: LCA results and circular KPI tool</t>
   </si>
@@ -96,7 +96,7 @@
     <t xml:space="preserve">Charts - environmental profile (radar), change vs polyculture, N and P fate, KPI targets met, margin to target. All live.</t>
   </si>
   <si>
-    <t xml:space="preserve">Figures - the report figures from make_charts.py as static images (key numbers, KPI framework, scorecard and more).</t>
+    <t xml:space="preserve">Figures - the report figures from make_charts.py as static images, each with its data table (live formulas) on the right.</t>
   </si>
   <si>
     <t xml:space="preserve">Data checks - cross-checks between the report tables (two findings are flagged on purpose).</t>
@@ -1137,34 +1137,160 @@
     <t xml:space="preserve">C6 Feed share of global warming</t>
   </si>
   <si>
-    <t xml:space="preserve">Figures - the report charts drawn by make_charts.py (static images; the Charts and Contribution analysis tabs are live)</t>
+    <t xml:space="preserve">Figures - the report charts drawn by make_charts.py, each with its data table on the right</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The pictures are static (published values). The tables next to them are live formulas, so they update when you change an input.</t>
   </si>
   <si>
     <t xml:space="preserve">00_key_numbers.png</t>
   </si>
   <si>
+    <t xml:space="preserve">Data: key numbers (per tonne of fish + oyster)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eutrophication vs fish-only pond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feed nitrogen kept in products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Global warming vs fish-only pond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of global warming from feed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Land competition vs fish-only pond</t>
+  </si>
+  <si>
     <t xml:space="preserve">01_change_vs_fish_pond.png</t>
   </si>
   <si>
+    <t xml:space="preserve">Data: change per tonne against the fish-only pond</t>
+  </si>
+  <si>
     <t xml:space="preserve">02_global_warming_by_process.png</t>
   </si>
   <si>
+    <t xml:space="preserve">Data: global warming by process, kg CO2-eq per tonne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy (pumping, aeration)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feed share of total</t>
+  </si>
+  <si>
     <t xml:space="preserve">03_nitrogen_fate.png</t>
   </si>
   <si>
+    <t xml:space="preserve">Data: fate of the feed nitrogen, kg N per tonne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">released to water (net; negative = uptake)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kept in products (N use efficiency)</t>
+  </si>
+  <si>
     <t xml:space="preserve">04_process_heatmap.png</t>
   </si>
   <si>
+    <t xml:space="preserve">Data: share of each impact per process - Semi-intensive pond IMTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data: share of each impact per process - Semi-extensive pond IMTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data: share of each impact per process - Semi-intensive fish polyculture</t>
+  </si>
+  <si>
     <t xml:space="preserve">05_kpi_scorecard.png</t>
   </si>
   <si>
+    <t xml:space="preserve">Data: KPI scorecard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E1 Global warming (kg CO2-eq/t)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E2 Cumulative energy demand (MJ-eq/t)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E3 Net primary production use (kg C/t)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E4 Acidification (kg SO2-eq/t)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E5 Eutrophication (kg PO4-eq/t)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E6 Land competition (m2a/t)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E7 Water dependence (m3/t)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1 Nitrogen use efficiency (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2 Phosphorus use efficiency (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3 Net N released to water (kg N/t)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4 Fish feed conversion ratio (kg/kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5 Share of non-fed (extractive) biomass (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C6 Feed share of global warming (%)</t>
+  </si>
+  <si>
     <t xml:space="preserve">06_environmental_profile.png</t>
   </si>
   <si>
+    <t xml:space="preserve">Data: each impact as % of the fish-only pond</t>
+  </si>
+  <si>
     <t xml:space="preserve">07_kpi_framework.png</t>
   </si>
   <si>
+    <t xml:space="preserve">Data: the framework steps with this workbook's numbers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Data: fish + oyster gain per pond, kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Scale: factor to 1 t = 1,000 / gain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 KPI example: N in feed per pond, kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 KPI example: N use efficiency (C1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 Target: improvement vs fish-only pond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 Score: targets met</t>
+  </si>
+  <si>
     <t xml:space="preserve">08_kpi_distance_to_target.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data: margin to target (positive = met; not capped)</t>
   </si>
   <si>
     <t xml:space="preserve">Data checks - do the report's tables agree with each other?</t>
@@ -1276,7 +1402,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="14">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.0#"/>
     <numFmt numFmtId="166" formatCode="#,##0.00##"/>
@@ -1290,6 +1416,7 @@
     <numFmt numFmtId="174" formatCode="\+0%;\-0%;0%"/>
     <numFmt numFmtId="175" formatCode="0.0"/>
     <numFmt numFmtId="176" formatCode="0"/>
+    <numFmt numFmtId="177" formatCode="0.000"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -1477,7 +1604,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1631,6 +1758,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="176" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2772,11 +2903,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="56045774"/>
-        <c:axId val="21160797"/>
+        <c:axId val="50001437"/>
+        <c:axId val="18661180"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="56045774"/>
+        <c:axId val="50001437"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2842,7 +2973,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21160797"/>
+        <c:crossAx val="18661180"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2850,7 +2981,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="21160797"/>
+        <c:axId val="18661180"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2927,7 +3058,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56045774"/>
+        <c:crossAx val="50001437"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3762,11 +3893,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="77862028"/>
-        <c:axId val="84166361"/>
+        <c:axId val="4229149"/>
+        <c:axId val="86793802"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="77862028"/>
+        <c:axId val="4229149"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3798,7 +3929,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84166361"/>
+        <c:crossAx val="86793802"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3806,7 +3937,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="84166361"/>
+        <c:axId val="86793802"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3882,7 +4013,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77862028"/>
+        <c:crossAx val="4229149"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4197,11 +4328,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="767186"/>
-        <c:axId val="77639614"/>
+        <c:axId val="95266752"/>
+        <c:axId val="57438052"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="767186"/>
+        <c:axId val="95266752"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4233,7 +4364,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77639614"/>
+        <c:crossAx val="57438052"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4241,7 +4372,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77639614"/>
+        <c:axId val="57438052"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4317,7 +4448,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="767186"/>
+        <c:crossAx val="95266752"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5136,11 +5267,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="41047730"/>
-        <c:axId val="79583683"/>
+        <c:axId val="41504961"/>
+        <c:axId val="32754121"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="41047730"/>
+        <c:axId val="41504961"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5172,7 +5303,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79583683"/>
+        <c:crossAx val="32754121"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5180,7 +5311,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79583683"/>
+        <c:axId val="32754121"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5256,7 +5387,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41047730"/>
+        <c:crossAx val="41504961"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5445,11 +5576,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="13838152"/>
-        <c:axId val="92164016"/>
+        <c:axId val="70834616"/>
+        <c:axId val="98198337"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="13838152"/>
+        <c:axId val="70834616"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5481,7 +5612,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92164016"/>
+        <c:crossAx val="98198337"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5489,7 +5620,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="92164016"/>
+        <c:axId val="98198337"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5565,7 +5696,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13838152"/>
+        <c:crossAx val="70834616"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5976,11 +6107,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="69912052"/>
-        <c:axId val="86985931"/>
+        <c:axId val="34399479"/>
+        <c:axId val="60988753"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="69912052"/>
+        <c:axId val="34399479"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -6009,7 +6140,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86985931"/>
+        <c:crossAx val="60988753"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6017,7 +6148,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86985931"/>
+        <c:axId val="60988753"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="2.5"/>
@@ -6061,7 +6192,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69912052"/>
+        <c:crossAx val="34399479"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.5"/>
@@ -6381,11 +6512,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="97262705"/>
-        <c:axId val="49391045"/>
+        <c:axId val="99213230"/>
+        <c:axId val="5326458"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="97262705"/>
+        <c:axId val="99213230"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -6417,7 +6548,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49391045"/>
+        <c:crossAx val="5326458"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6425,7 +6556,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="49391045"/>
+        <c:axId val="5326458"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1.5"/>
@@ -6469,7 +6600,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97262705"/>
+        <c:crossAx val="99213230"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6826,11 +6957,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="63024862"/>
-        <c:axId val="5107328"/>
+        <c:axId val="31614319"/>
+        <c:axId val="78605771"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="63024862"/>
+        <c:axId val="31614319"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -6862,7 +6993,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5107328"/>
+        <c:crossAx val="78605771"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6870,7 +7001,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5107328"/>
+        <c:axId val="78605771"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6946,7 +7077,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63024862"/>
+        <c:crossAx val="31614319"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7303,11 +7434,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="71549911"/>
-        <c:axId val="44296819"/>
+        <c:axId val="68352169"/>
+        <c:axId val="58276591"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="71549911"/>
+        <c:axId val="68352169"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -7339,7 +7470,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44296819"/>
+        <c:crossAx val="58276591"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7347,7 +7478,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44296819"/>
+        <c:axId val="58276591"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7423,7 +7554,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71549911"/>
+        <c:crossAx val="68352169"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7694,11 +7825,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="57318624"/>
-        <c:axId val="92584662"/>
+        <c:axId val="25647902"/>
+        <c:axId val="90124289"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="57318624"/>
+        <c:axId val="25647902"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7730,7 +7861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92584662"/>
+        <c:crossAx val="90124289"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7738,7 +7869,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="92584662"/>
+        <c:axId val="90124289"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -7816,7 +7947,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57318624"/>
+        <c:crossAx val="25647902"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -8333,11 +8464,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="829933"/>
-        <c:axId val="93632547"/>
+        <c:axId val="18918071"/>
+        <c:axId val="34676297"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="829933"/>
+        <c:axId val="18918071"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -8369,7 +8500,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93632547"/>
+        <c:crossAx val="34676297"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8377,7 +8508,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93632547"/>
+        <c:axId val="34676297"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1.5"/>
@@ -8421,7 +8552,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="829933"/>
+        <c:crossAx val="18918071"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9512,11 +9643,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="5311162"/>
-        <c:axId val="71801388"/>
+        <c:axId val="69575688"/>
+        <c:axId val="58039743"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="5311162"/>
+        <c:axId val="69575688"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -9582,7 +9713,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71801388"/>
+        <c:crossAx val="58039743"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9590,7 +9721,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71801388"/>
+        <c:axId val="58039743"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -9667,7 +9798,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5311162"/>
+        <c:crossAx val="69575688"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -10758,11 +10889,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="10377400"/>
-        <c:axId val="57017701"/>
+        <c:axId val="65251218"/>
+        <c:axId val="87828508"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="10377400"/>
+        <c:axId val="65251218"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -10828,7 +10959,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57017701"/>
+        <c:crossAx val="87828508"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10836,7 +10967,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="57017701"/>
+        <c:axId val="87828508"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -10913,7 +11044,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10377400"/>
+        <c:crossAx val="65251218"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -11748,11 +11879,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="38983969"/>
-        <c:axId val="2971029"/>
+        <c:axId val="17099210"/>
+        <c:axId val="94018332"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="38983969"/>
+        <c:axId val="17099210"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11784,7 +11915,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2971029"/>
+        <c:crossAx val="94018332"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -11792,7 +11923,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2971029"/>
+        <c:axId val="94018332"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11868,7 +11999,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38983969"/>
+        <c:crossAx val="17099210"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -12703,11 +12834,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="6923214"/>
-        <c:axId val="82723245"/>
+        <c:axId val="51264480"/>
+        <c:axId val="79516288"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="6923214"/>
+        <c:axId val="51264480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12739,7 +12870,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82723245"/>
+        <c:crossAx val="79516288"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -12747,7 +12878,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="82723245"/>
+        <c:axId val="79516288"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12823,7 +12954,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6923214"/>
+        <c:crossAx val="51264480"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13658,11 +13789,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="85957270"/>
-        <c:axId val="5751986"/>
+        <c:axId val="61173992"/>
+        <c:axId val="61379751"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="85957270"/>
+        <c:axId val="61173992"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13694,7 +13825,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5751986"/>
+        <c:crossAx val="61379751"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13702,7 +13833,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5751986"/>
+        <c:axId val="61379751"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13778,7 +13909,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85957270"/>
+        <c:crossAx val="61173992"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -14613,11 +14744,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="64129379"/>
-        <c:axId val="27650420"/>
+        <c:axId val="77845155"/>
+        <c:axId val="66944730"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="64129379"/>
+        <c:axId val="77845155"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14649,7 +14780,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27650420"/>
+        <c:crossAx val="66944730"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -14657,7 +14788,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="27650420"/>
+        <c:axId val="66944730"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14733,7 +14864,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64129379"/>
+        <c:crossAx val="77845155"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -15568,11 +15699,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="91778809"/>
-        <c:axId val="39518716"/>
+        <c:axId val="51204528"/>
+        <c:axId val="347616"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="91778809"/>
+        <c:axId val="51204528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -15604,7 +15735,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39518716"/>
+        <c:crossAx val="347616"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -15612,7 +15743,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="39518716"/>
+        <c:axId val="347616"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -15688,7 +15819,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91778809"/>
+        <c:crossAx val="51204528"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -16523,11 +16654,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="9215129"/>
-        <c:axId val="78194370"/>
+        <c:axId val="69139599"/>
+        <c:axId val="38816603"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="9215129"/>
+        <c:axId val="69139599"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16559,7 +16690,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78194370"/>
+        <c:crossAx val="38816603"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -16567,7 +16698,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78194370"/>
+        <c:axId val="38816603"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16643,7 +16774,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9215129"/>
+        <c:crossAx val="69139599"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -17291,14 +17422,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>160920</xdr:rowOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>160560</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>11160</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
+      <xdr:rowOff>39240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -17311,7 +17442,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="762120"/>
+          <a:off x="0" y="952560"/>
           <a:ext cx="8572320" cy="3428640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -17329,13 +17460,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
+      <xdr:rowOff>39600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>11160</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>160200</xdr:rowOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>79200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -17348,7 +17479,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="4952880"/>
+          <a:off x="0" y="5143680"/>
           <a:ext cx="8572320" cy="4571640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -17365,14 +17496,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>79200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>11160</xdr:colOff>
-      <xdr:row>78</xdr:row>
-      <xdr:rowOff>160200</xdr:rowOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>147960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -17385,7 +17516,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="10287000"/>
+          <a:off x="0" y="10477440"/>
           <a:ext cx="8572320" cy="4762080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -17402,14 +17533,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>82</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>148680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>11160</xdr:colOff>
-      <xdr:row>104</xdr:row>
-      <xdr:rowOff>150840</xdr:rowOff>
+      <xdr:row>100</xdr:row>
+      <xdr:rowOff>17280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -17422,7 +17553,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="15811560"/>
+          <a:off x="0" y="16002000"/>
           <a:ext cx="8572320" cy="4181040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -17439,14 +17570,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>107</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>27360</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>11160</xdr:colOff>
-      <xdr:row>126</xdr:row>
-      <xdr:rowOff>36360</xdr:rowOff>
+      <xdr:row>121</xdr:row>
+      <xdr:rowOff>93600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -17459,7 +17590,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="20574000"/>
+          <a:off x="0" y="20764440"/>
           <a:ext cx="8572320" cy="3495240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -17476,14 +17607,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>129</xdr:row>
-      <xdr:rowOff>160920</xdr:rowOff>
+      <xdr:row>140</xdr:row>
+      <xdr:rowOff>27360</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>11160</xdr:colOff>
-      <xdr:row>161</xdr:row>
-      <xdr:rowOff>17280</xdr:rowOff>
+      <xdr:row>170</xdr:row>
+      <xdr:rowOff>114120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -17496,7 +17627,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="24765120"/>
+          <a:off x="0" y="27812880"/>
           <a:ext cx="8572320" cy="5952600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -17513,14 +17644,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>164</xdr:row>
-      <xdr:rowOff>160920</xdr:rowOff>
+      <xdr:row>174</xdr:row>
+      <xdr:rowOff>67320</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>11160</xdr:colOff>
-      <xdr:row>202</xdr:row>
-      <xdr:rowOff>150840</xdr:rowOff>
+      <xdr:row>210</xdr:row>
+      <xdr:rowOff>126720</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -17533,7 +17664,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="31432680"/>
+          <a:off x="0" y="34480440"/>
           <a:ext cx="8572320" cy="7229160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -17550,14 +17681,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>205</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
+      <xdr:row>213</xdr:row>
+      <xdr:rowOff>136440</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>11160</xdr:colOff>
-      <xdr:row>224</xdr:row>
-      <xdr:rowOff>102960</xdr:rowOff>
+      <xdr:row>230</xdr:row>
+      <xdr:rowOff>147960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -17570,7 +17701,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="39242880"/>
+          <a:off x="0" y="42291000"/>
           <a:ext cx="8572320" cy="3561840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -17587,14 +17718,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>227</xdr:row>
-      <xdr:rowOff>160560</xdr:rowOff>
+      <xdr:row>234</xdr:row>
+      <xdr:rowOff>15480</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>11160</xdr:colOff>
-      <xdr:row>258</xdr:row>
-      <xdr:rowOff>27000</xdr:rowOff>
+      <xdr:row>262</xdr:row>
+      <xdr:rowOff>141480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -17607,7 +17738,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="43434000"/>
+          <a:off x="0" y="46482120"/>
           <a:ext cx="8572320" cy="5771880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -19855,8 +19986,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A228"/>
+  <dimension ref="A1:W259"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="17" style="0" width="14"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -19868,52 +20003,2456 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="2" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P6" s="3" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="2" t="s">
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P7" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P8" s="31" t="s">
+        <v>335</v>
+      </c>
+      <c r="Q8" s="21" t="n">
+        <f aca="false">Comparison!C9</f>
+        <v>26</v>
+      </c>
+      <c r="R8" s="21" t="n">
+        <f aca="false">Comparison!D9</f>
+        <v>2</v>
+      </c>
+      <c r="S8" s="21" t="n">
+        <f aca="false">Comparison!E9</f>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P9" s="31" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="2" t="s">
+      <c r="Q9" s="23" t="n">
+        <f aca="false">Comparison!C9/Comparison!$E9-1</f>
+        <v>-0.573770491803279</v>
+      </c>
+      <c r="R9" s="23" t="n">
+        <f aca="false">Comparison!D9/Comparison!$E9-1</f>
+        <v>-0.967213114754098</v>
+      </c>
+      <c r="S9" s="23" t="n">
+        <f aca="false">Comparison!E9/Comparison!$E9-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P10" s="31" t="s">
         <v>372</v>
       </c>
+      <c r="Q10" s="23" t="n">
+        <f aca="false">'Nutrient balance'!C13</f>
+        <v>0.469758878127522</v>
+      </c>
+      <c r="R10" s="23" t="n">
+        <f aca="false">'Nutrient balance'!D13</f>
+        <v>1.1060393258427</v>
+      </c>
+      <c r="S10" s="23" t="n">
+        <f aca="false">'Nutrient balance'!E13</f>
+        <v>0.201757240481614</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P11" s="31" t="s">
+        <v>334</v>
+      </c>
+      <c r="Q11" s="21" t="n">
+        <f aca="false">Comparison!C5</f>
+        <v>2801</v>
+      </c>
+      <c r="R11" s="21" t="n">
+        <f aca="false">Comparison!D5</f>
+        <v>1255</v>
+      </c>
+      <c r="S11" s="21" t="n">
+        <f aca="false">Comparison!E5</f>
+        <v>2836</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P12" s="31" t="s">
+        <v>373</v>
+      </c>
+      <c r="Q12" s="23" t="n">
+        <f aca="false">Comparison!C5/Comparison!$E5-1</f>
+        <v>-0.0123413258110014</v>
+      </c>
+      <c r="R12" s="23" t="n">
+        <f aca="false">Comparison!D5/Comparison!$E5-1</f>
+        <v>-0.557475317348378</v>
+      </c>
+      <c r="S12" s="23" t="n">
+        <f aca="false">Comparison!E5/Comparison!$E5-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P13" s="31" t="s">
+        <v>374</v>
+      </c>
+      <c r="Q13" s="23" t="n">
+        <f aca="false">'LCIA (Annex 1)'!C14/'LCIA (Annex 1)'!C18</f>
+        <v>0.553016779721528</v>
+      </c>
+      <c r="R13" s="23" t="n">
+        <f aca="false">'LCIA (Annex 1)'!D14/'LCIA (Annex 1)'!D18</f>
+        <v>0.58406374501992</v>
+      </c>
+      <c r="S13" s="23" t="n">
+        <f aca="false">'LCIA (Annex 1)'!E14/'LCIA (Annex 1)'!E18</f>
+        <v>0.660437235543018</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P14" s="31" t="s">
+        <v>337</v>
+      </c>
+      <c r="Q14" s="21" t="n">
+        <f aca="false">Comparison!C10</f>
+        <v>2946</v>
+      </c>
+      <c r="R14" s="21" t="n">
+        <f aca="false">Comparison!D10</f>
+        <v>4885</v>
+      </c>
+      <c r="S14" s="21" t="n">
+        <f aca="false">Comparison!E10</f>
+        <v>2379</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P15" s="31" t="s">
+        <v>375</v>
+      </c>
+      <c r="Q15" s="23" t="n">
+        <f aca="false">Comparison!C10/Comparison!$E10-1</f>
+        <v>0.238335435056747</v>
+      </c>
+      <c r="R15" s="23" t="n">
+        <f aca="false">Comparison!D10/Comparison!$E10-1</f>
+        <v>1.05338377469525</v>
+      </c>
+      <c r="S15" s="23" t="n">
+        <f aca="false">Comparison!E10/Comparison!$E10-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P28" s="3" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P29" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="Q29" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="R29" s="5" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P30" s="31" t="s">
+        <v>286</v>
+      </c>
+      <c r="Q30" s="27" t="n">
+        <f aca="false">Comparison!F5</f>
+        <v>-0.0123413258110014</v>
+      </c>
+      <c r="R30" s="27" t="n">
+        <f aca="false">Comparison!G5</f>
+        <v>-0.557475317348378</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P31" s="31" t="s">
+        <v>292</v>
+      </c>
+      <c r="Q31" s="27" t="n">
+        <f aca="false">Comparison!F6</f>
+        <v>-0.0978007347567995</v>
+      </c>
+      <c r="R31" s="27" t="n">
+        <f aca="false">Comparison!G6</f>
+        <v>-0.808833098091034</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P32" s="31" t="s">
+        <v>295</v>
+      </c>
+      <c r="Q32" s="27" t="n">
+        <f aca="false">Comparison!F7</f>
+        <v>-0.152128176080272</v>
+      </c>
+      <c r="R32" s="27" t="n">
+        <f aca="false">Comparison!G7</f>
+        <v>-0.643793494092895</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P33" s="31" t="s">
+        <v>298</v>
+      </c>
+      <c r="Q33" s="27" t="n">
+        <f aca="false">Comparison!F8</f>
+        <v>-0.0666666666666667</v>
+      </c>
+      <c r="R33" s="27" t="n">
+        <f aca="false">Comparison!G8</f>
+        <v>-0.866666666666667</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P34" s="31" t="s">
+        <v>301</v>
+      </c>
+      <c r="Q34" s="27" t="n">
+        <f aca="false">Comparison!F9</f>
+        <v>-0.573770491803279</v>
+      </c>
+      <c r="R34" s="27" t="n">
+        <f aca="false">Comparison!G9</f>
+        <v>-0.967213114754098</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P35" s="31" t="s">
+        <v>304</v>
+      </c>
+      <c r="Q35" s="27" t="n">
+        <f aca="false">Comparison!F10</f>
+        <v>0.238335435056747</v>
+      </c>
+      <c r="R35" s="27" t="n">
+        <f aca="false">Comparison!G10</f>
+        <v>1.05338377469525</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P36" s="31" t="s">
+        <v>307</v>
+      </c>
+      <c r="Q36" s="27" t="n">
+        <f aca="false">Comparison!F11</f>
+        <v>-0.583106447295434</v>
+      </c>
+      <c r="R36" s="27" t="n">
+        <f aca="false">Comparison!G11</f>
+        <v>-0.705622363244971</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P56" s="3" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P57" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q57" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="R57" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="S57" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P58" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q58" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!C14</f>
+        <v>1549</v>
+      </c>
+      <c r="R58" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!D14</f>
+        <v>733</v>
+      </c>
+      <c r="S58" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!E14</f>
+        <v>1873</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P59" s="31" t="s">
+        <v>380</v>
+      </c>
+      <c r="Q59" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!C15</f>
+        <v>325</v>
+      </c>
+      <c r="R59" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!D15</f>
+        <v>208</v>
+      </c>
+      <c r="S59" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!E15</f>
+        <v>379</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P60" s="31" t="s">
+        <v>381</v>
+      </c>
+      <c r="Q60" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!C7</f>
+        <v>330</v>
+      </c>
+      <c r="R60" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!D7</f>
+        <v>6</v>
+      </c>
+      <c r="S60" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!E7</f>
+        <v>474</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P61" s="31" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q61" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!C12</f>
+        <v>386</v>
+      </c>
+      <c r="R61" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!D12</f>
+        <v>228</v>
+      </c>
+      <c r="S61" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!E12</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P62" s="31" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q62" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!C6+'LCIA (Annex 1)'!C9+'LCIA (Annex 1)'!C11+'LCIA (Annex 1)'!C13</f>
+        <v>212</v>
+      </c>
+      <c r="R62" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!D6+'LCIA (Annex 1)'!D9+'LCIA (Annex 1)'!D11+'LCIA (Annex 1)'!D13</f>
+        <v>79</v>
+      </c>
+      <c r="S62" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!E6+'LCIA (Annex 1)'!E9+'LCIA (Annex 1)'!E11+'LCIA (Annex 1)'!E13</f>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P63" s="31" t="s">
+        <v>216</v>
+      </c>
+      <c r="Q63" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!C18</f>
+        <v>2801</v>
+      </c>
+      <c r="R63" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!D18</f>
+        <v>1255</v>
+      </c>
+      <c r="S63" s="21" t="n">
+        <f aca="false">'LCIA (Annex 1)'!E18</f>
+        <v>2836</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P64" s="31" t="s">
+        <v>382</v>
+      </c>
+      <c r="Q64" s="23" t="n">
+        <f aca="false">'LCIA (Annex 1)'!C14/'LCIA (Annex 1)'!C18</f>
+        <v>0.553016779721528</v>
+      </c>
+      <c r="R64" s="23" t="n">
+        <f aca="false">'LCIA (Annex 1)'!D14/'LCIA (Annex 1)'!D18</f>
+        <v>0.58406374501992</v>
+      </c>
+      <c r="S64" s="23" t="n">
+        <f aca="false">'LCIA (Annex 1)'!E14/'LCIA (Annex 1)'!E18</f>
+        <v>0.660437235543018</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P85" s="3" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P86" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q86" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="R86" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="S86" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P87" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q87" s="16" t="n">
+        <f aca="false">'Nutrient balance'!C8*Inventory!C25</f>
+        <v>103.233197721725</v>
+      </c>
+      <c r="R87" s="16" t="n">
+        <f aca="false">'Nutrient balance'!D8*Inventory!D25</f>
+        <v>35.8238993710692</v>
+      </c>
+      <c r="S87" s="16" t="n">
+        <f aca="false">'Nutrient balance'!E8*Inventory!E25</f>
+        <v>120.175981750041</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P88" s="31" t="s">
+        <v>345</v>
+      </c>
+      <c r="Q88" s="16" t="n">
+        <f aca="false">'Nutrient balance'!C9*Inventory!C25</f>
+        <v>23.5964198535395</v>
+      </c>
+      <c r="R88" s="16" t="n">
+        <f aca="false">'Nutrient balance'!D9*Inventory!D25</f>
+        <v>28.3018867924528</v>
+      </c>
+      <c r="S88" s="16" t="n">
+        <f aca="false">'Nutrient balance'!E9*Inventory!E25</f>
+        <v>24.246374450057</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P89" s="31" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q89" s="16" t="n">
+        <f aca="false">'Nutrient balance'!C10*Inventory!C25</f>
+        <v>24.8982912937347</v>
+      </c>
+      <c r="R89" s="16" t="n">
+        <f aca="false">'Nutrient balance'!D10*Inventory!D25</f>
+        <v>11.3207547169811</v>
+      </c>
+      <c r="S89" s="16" t="n">
+        <f aca="false">'Nutrient balance'!E10*Inventory!E25</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P90" s="31" t="s">
+        <v>385</v>
+      </c>
+      <c r="Q90" s="16" t="n">
+        <f aca="false">'Nutrient balance'!C11*Inventory!C25</f>
+        <v>54.7384865744508</v>
+      </c>
+      <c r="R90" s="16" t="n">
+        <f aca="false">'Nutrient balance'!D11*Inventory!D25</f>
+        <v>-3.79874213836478</v>
+      </c>
+      <c r="S90" s="16" t="n">
+        <f aca="false">'Nutrient balance'!E11*Inventory!E25</f>
+        <v>95.9296072999837</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P91" s="31" t="s">
+        <v>386</v>
+      </c>
+      <c r="Q91" s="23" t="n">
+        <f aca="false">'Nutrient balance'!C13</f>
+        <v>0.469758878127522</v>
+      </c>
+      <c r="R91" s="23" t="n">
+        <f aca="false">'Nutrient balance'!D13</f>
+        <v>1.1060393258427</v>
+      </c>
+      <c r="S91" s="23" t="n">
+        <f aca="false">'Nutrient balance'!E13</f>
+        <v>0.201757240481614</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="2" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P110" s="3" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P111" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q111" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="R111" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="S111" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="T111" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="U111" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="V111" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="W111" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P112" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q112" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16))=0,0,('LCIA (Annex 1)'!C14)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16)))</f>
+        <v>0.552819414703783</v>
+      </c>
+      <c r="R112" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31))=0,0,('LCIA (Annex 1)'!C29)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31)))</f>
+        <v>0.233312622048642</v>
+      </c>
+      <c r="S112" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46))=0,0,('LCIA (Annex 1)'!C44)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46)))</f>
+        <v>0.994750906661577</v>
+      </c>
+      <c r="T112" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61))=0,0,('LCIA (Annex 1)'!C59)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61)))</f>
+        <v>0.19047619047619</v>
+      </c>
+      <c r="U112" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76))=0,0,('LCIA (Annex 1)'!C74)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76)))</f>
+        <v>0.307692307692308</v>
+      </c>
+      <c r="V112" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91))=0,0,('LCIA (Annex 1)'!C89)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91)))</f>
+        <v>0.659198913781399</v>
+      </c>
+      <c r="W112" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106))=0,0,('LCIA (Annex 1)'!C104)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106)))</f>
+        <v>0.000286863483499246</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P113" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q113" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16))=0,0,('LCIA (Annex 1)'!C10)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16)))</f>
+        <v>0</v>
+      </c>
+      <c r="R113" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31))=0,0,('LCIA (Annex 1)'!C25)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31)))</f>
+        <v>0</v>
+      </c>
+      <c r="S113" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46))=0,0,('LCIA (Annex 1)'!C40)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T113" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61))=0,0,('LCIA (Annex 1)'!C55)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61)))</f>
+        <v>0.595238095238095</v>
+      </c>
+      <c r="U113" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76))=0,0,('LCIA (Annex 1)'!C70)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76)))</f>
+        <v>0.615384615384615</v>
+      </c>
+      <c r="V113" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91))=0,0,('LCIA (Annex 1)'!C85)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91)))</f>
+        <v>0</v>
+      </c>
+      <c r="W113" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106))=0,0,('LCIA (Annex 1)'!C100)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P114" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q114" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16))=0,0,('LCIA (Annex 1)'!C7)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16)))</f>
+        <v>0.117773019271949</v>
+      </c>
+      <c r="R114" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31))=0,0,('LCIA (Annex 1)'!C22)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31)))</f>
+        <v>0.507322918515889</v>
+      </c>
+      <c r="S114" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46))=0,0,('LCIA (Annex 1)'!C37)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T114" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61))=0,0,('LCIA (Annex 1)'!C52)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61)))</f>
+        <v>0.0476190476190476</v>
+      </c>
+      <c r="U114" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76))=0,0,('LCIA (Annex 1)'!C67)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76)))</f>
+        <v>0.0384615384615385</v>
+      </c>
+      <c r="V114" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91))=0,0,('LCIA (Annex 1)'!C82)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91)))</f>
+        <v>0.00271554650373388</v>
+      </c>
+      <c r="W114" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106))=0,0,('LCIA (Annex 1)'!C97)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106)))</f>
+        <v>0.000231932178148327</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P115" s="31" t="s">
+        <v>213</v>
+      </c>
+      <c r="Q115" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16))=0,0,('LCIA (Annex 1)'!C15)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16)))</f>
+        <v>0.11598857958601</v>
+      </c>
+      <c r="R115" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31))=0,0,('LCIA (Annex 1)'!C30)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31)))</f>
+        <v>0.0608357003372981</v>
+      </c>
+      <c r="S115" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46))=0,0,('LCIA (Annex 1)'!C45)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T115" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61))=0,0,('LCIA (Annex 1)'!C60)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61)))</f>
+        <v>0.0476190476190476</v>
+      </c>
+      <c r="U115" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76))=0,0,('LCIA (Annex 1)'!C75)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V115" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91))=0,0,('LCIA (Annex 1)'!C90)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91)))</f>
+        <v>0.00135777325186694</v>
+      </c>
+      <c r="W115" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106))=0,0,('LCIA (Annex 1)'!C105)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106)))</f>
+        <v>1.83104351169732E-005</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P116" s="31" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q116" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16))=0,0,('LCIA (Annex 1)'!C12)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16)))</f>
+        <v>0.137758743754461</v>
+      </c>
+      <c r="R116" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31))=0,0,('LCIA (Annex 1)'!C27)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31)))</f>
+        <v>0.155589827800462</v>
+      </c>
+      <c r="S116" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46))=0,0,('LCIA (Annex 1)'!C42)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T116" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61))=0,0,('LCIA (Annex 1)'!C57)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61)))</f>
+        <v>0.0714285714285714</v>
+      </c>
+      <c r="U116" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76))=0,0,('LCIA (Annex 1)'!C72)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76)))</f>
+        <v>0.0384615384615385</v>
+      </c>
+      <c r="V116" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91))=0,0,('LCIA (Annex 1)'!C87)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91)))</f>
+        <v>0.00203665987780041</v>
+      </c>
+      <c r="W116" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106))=0,0,('LCIA (Annex 1)'!C102)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106)))</f>
+        <v>3.66208702339463E-005</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P117" s="31" t="s">
+        <v>239</v>
+      </c>
+      <c r="Q117" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16))=0,0,('LCIA (Annex 1)'!C16)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16)))</f>
+        <v>0</v>
+      </c>
+      <c r="R117" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31))=0,0,('LCIA (Annex 1)'!C31)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31)))</f>
+        <v>0</v>
+      </c>
+      <c r="S117" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46))=0,0,('LCIA (Annex 1)'!C46)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T117" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61))=0,0,('LCIA (Annex 1)'!C61)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U117" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76))=0,0,('LCIA (Annex 1)'!C76)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V117" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91))=0,0,('LCIA (Annex 1)'!C91)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91)))</f>
+        <v>0.319416157501697</v>
+      </c>
+      <c r="W117" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106))=0,0,('LCIA (Annex 1)'!C106)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106)))</f>
+        <v>0.496432516891376</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P118" s="31" t="s">
+        <v>206</v>
+      </c>
+      <c r="Q118" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16))=0,0,('LCIA (Annex 1)'!C8)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16)))</f>
+        <v>0</v>
+      </c>
+      <c r="R118" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31))=0,0,('LCIA (Annex 1)'!C23)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31)))</f>
+        <v>0</v>
+      </c>
+      <c r="S118" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46))=0,0,('LCIA (Annex 1)'!C38)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T118" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61))=0,0,('LCIA (Annex 1)'!C53)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U118" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76))=0,0,('LCIA (Annex 1)'!C68)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V118" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91))=0,0,('LCIA (Annex 1)'!C83)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91)))</f>
+        <v>0</v>
+      </c>
+      <c r="W118" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106))=0,0,('LCIA (Annex 1)'!C98)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106)))</f>
+        <v>0.502078234385777</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P119" s="31" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q119" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16))=0,0,('LCIA (Annex 1)'!C6+'LCIA (Annex 1)'!C9+'LCIA (Annex 1)'!C11+'LCIA (Annex 1)'!C13)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C6:C16)))</f>
+        <v>0.0756602426837973</v>
+      </c>
+      <c r="R119" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31))=0,0,('LCIA (Annex 1)'!C21+'LCIA (Annex 1)'!C24+'LCIA (Annex 1)'!C26+'LCIA (Annex 1)'!C28)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C21:C31)))</f>
+        <v>0.0429389312977099</v>
+      </c>
+      <c r="S119" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46))=0,0,('LCIA (Annex 1)'!C36+'LCIA (Annex 1)'!C39+'LCIA (Annex 1)'!C41+'LCIA (Annex 1)'!C43)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C36:C46)))</f>
+        <v>0.00524909333842336</v>
+      </c>
+      <c r="T119" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61))=0,0,('LCIA (Annex 1)'!C51+'LCIA (Annex 1)'!C54+'LCIA (Annex 1)'!C56+'LCIA (Annex 1)'!C58)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C51:C61)))</f>
+        <v>0.0476190476190476</v>
+      </c>
+      <c r="U119" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76))=0,0,('LCIA (Annex 1)'!C66+'LCIA (Annex 1)'!C69+'LCIA (Annex 1)'!C71+'LCIA (Annex 1)'!C73)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C66:C76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V119" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91))=0,0,('LCIA (Annex 1)'!C81+'LCIA (Annex 1)'!C84+'LCIA (Annex 1)'!C86+'LCIA (Annex 1)'!C88)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C81:C91)))</f>
+        <v>0.0152749490835031</v>
+      </c>
+      <c r="W119" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106))=0,0,('LCIA (Annex 1)'!C96+'LCIA (Annex 1)'!C99+'LCIA (Annex 1)'!C101+'LCIA (Annex 1)'!C103)/SUMPRODUCT(ABS('LCIA (Annex 1)'!C96:C106)))</f>
+        <v>0.000915521755848658</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P121" s="3" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P122" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q122" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="R122" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="S122" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="T122" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="U122" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="V122" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="W122" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P123" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q123" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16))=0,0,('LCIA (Annex 1)'!D14)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16)))</f>
+        <v>0.584529505582137</v>
+      </c>
+      <c r="R123" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31))=0,0,('LCIA (Annex 1)'!D29)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31)))</f>
+        <v>0.413677540975022</v>
+      </c>
+      <c r="S123" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46))=0,0,('LCIA (Annex 1)'!D44)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46)))</f>
+        <v>0.991594729668333</v>
+      </c>
+      <c r="T123" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61))=0,0,('LCIA (Annex 1)'!D59)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61)))</f>
+        <v>0.6</v>
+      </c>
+      <c r="U123" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76))=0,0,('LCIA (Annex 1)'!D74)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76)))</f>
+        <v>0.75</v>
+      </c>
+      <c r="V123" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91))=0,0,('LCIA (Annex 1)'!D89)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91)))</f>
+        <v>0.135135135135135</v>
+      </c>
+      <c r="W123" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106))=0,0,('LCIA (Annex 1)'!D104)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106)))</f>
+        <v>0.000121010960135532</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P124" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q124" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16))=0,0,('LCIA (Annex 1)'!D10)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16)))</f>
+        <v>0</v>
+      </c>
+      <c r="R124" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31))=0,0,('LCIA (Annex 1)'!D25)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31)))</f>
+        <v>0</v>
+      </c>
+      <c r="S124" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46))=0,0,('LCIA (Annex 1)'!D40)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T124" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61))=0,0,('LCIA (Annex 1)'!D55)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U124" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76))=0,0,('LCIA (Annex 1)'!D70)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76)))</f>
+        <v>-0.25</v>
+      </c>
+      <c r="V124" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91))=0,0,('LCIA (Annex 1)'!D85)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91)))</f>
+        <v>0</v>
+      </c>
+      <c r="W124" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106))=0,0,('LCIA (Annex 1)'!D100)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P125" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q125" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16))=0,0,('LCIA (Annex 1)'!D7)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16)))</f>
+        <v>0.00478468899521531</v>
+      </c>
+      <c r="R125" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31))=0,0,('LCIA (Annex 1)'!D22)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31)))</f>
+        <v>0.00429386814682935</v>
+      </c>
+      <c r="S125" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46))=0,0,('LCIA (Annex 1)'!D37)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T125" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61))=0,0,('LCIA (Annex 1)'!D52)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U125" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76))=0,0,('LCIA (Annex 1)'!D67)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V125" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91))=0,0,('LCIA (Annex 1)'!D82)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91)))</f>
+        <v>0</v>
+      </c>
+      <c r="W125" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106))=0,0,('LCIA (Annex 1)'!D97)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P126" s="31" t="s">
+        <v>213</v>
+      </c>
+      <c r="Q126" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16))=0,0,('LCIA (Annex 1)'!D15)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16)))</f>
+        <v>0.165869218500797</v>
+      </c>
+      <c r="R126" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31))=0,0,('LCIA (Annex 1)'!D30)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31)))</f>
+        <v>0.183117767188564</v>
+      </c>
+      <c r="S126" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46))=0,0,('LCIA (Annex 1)'!D45)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T126" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61))=0,0,('LCIA (Annex 1)'!D60)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61)))</f>
+        <v>0.2</v>
+      </c>
+      <c r="U126" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76))=0,0,('LCIA (Annex 1)'!D75)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V126" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91))=0,0,('LCIA (Annex 1)'!D90)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91)))</f>
+        <v>0.000614250614250614</v>
+      </c>
+      <c r="W126" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106))=0,0,('LCIA (Annex 1)'!D105)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106)))</f>
+        <v>1.72872800193618E-005</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P127" s="31" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q127" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16))=0,0,('LCIA (Annex 1)'!D12)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16)))</f>
+        <v>0.181818181818182</v>
+      </c>
+      <c r="R127" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31))=0,0,('LCIA (Annex 1)'!D27)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31)))</f>
+        <v>0.327171807090119</v>
+      </c>
+      <c r="S127" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46))=0,0,('LCIA (Annex 1)'!D42)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T127" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61))=0,0,('LCIA (Annex 1)'!D57)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61)))</f>
+        <v>0.2</v>
+      </c>
+      <c r="U127" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76))=0,0,('LCIA (Annex 1)'!D72)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V127" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91))=0,0,('LCIA (Annex 1)'!D87)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91)))</f>
+        <v>0</v>
+      </c>
+      <c r="W127" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106))=0,0,('LCIA (Annex 1)'!D102)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106)))</f>
+        <v>4.32182000484044E-005</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P128" s="31" t="s">
+        <v>239</v>
+      </c>
+      <c r="Q128" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16))=0,0,('LCIA (Annex 1)'!D16)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16)))</f>
+        <v>0</v>
+      </c>
+      <c r="R128" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31))=0,0,('LCIA (Annex 1)'!D31)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31)))</f>
+        <v>0</v>
+      </c>
+      <c r="S128" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46))=0,0,('LCIA (Annex 1)'!D46)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T128" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61))=0,0,('LCIA (Annex 1)'!D61)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U128" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76))=0,0,('LCIA (Annex 1)'!D76)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V128" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91))=0,0,('LCIA (Annex 1)'!D91)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91)))</f>
+        <v>0.858722358722359</v>
+      </c>
+      <c r="W128" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106))=0,0,('LCIA (Annex 1)'!D106)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106)))</f>
+        <v>0.607621961760537</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P129" s="31" t="s">
+        <v>206</v>
+      </c>
+      <c r="Q129" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16))=0,0,('LCIA (Annex 1)'!D8)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16)))</f>
+        <v>0</v>
+      </c>
+      <c r="R129" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31))=0,0,('LCIA (Annex 1)'!D23)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31)))</f>
+        <v>0</v>
+      </c>
+      <c r="S129" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46))=0,0,('LCIA (Annex 1)'!D38)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T129" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61))=0,0,('LCIA (Annex 1)'!D53)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U129" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76))=0,0,('LCIA (Annex 1)'!D68)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V129" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91))=0,0,('LCIA (Annex 1)'!D83)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91)))</f>
+        <v>0</v>
+      </c>
+      <c r="W129" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106))=0,0,('LCIA (Annex 1)'!D98)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106)))</f>
+        <v>0.391323514158282</v>
+      </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="2" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A165" s="2" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A206" s="2" t="s">
-        <v>375</v>
+      <c r="P130" s="31" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q130" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16))=0,0,('LCIA (Annex 1)'!D6+'LCIA (Annex 1)'!D9+'LCIA (Annex 1)'!D11+'LCIA (Annex 1)'!D13)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D6:D16)))</f>
+        <v>0.0629984051036683</v>
+      </c>
+      <c r="R130" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31))=0,0,('LCIA (Annex 1)'!D21+'LCIA (Annex 1)'!D24+'LCIA (Annex 1)'!D26+'LCIA (Annex 1)'!D28)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D21:D31)))</f>
+        <v>0.0717390165994659</v>
+      </c>
+      <c r="S130" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46))=0,0,('LCIA (Annex 1)'!D36+'LCIA (Annex 1)'!D39+'LCIA (Annex 1)'!D41+'LCIA (Annex 1)'!D43)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D36:D46)))</f>
+        <v>0.00840527033166742</v>
+      </c>
+      <c r="T130" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61))=0,0,('LCIA (Annex 1)'!D51+'LCIA (Annex 1)'!D54+'LCIA (Annex 1)'!D56+'LCIA (Annex 1)'!D58)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D51:D61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U130" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76))=0,0,('LCIA (Annex 1)'!D66+'LCIA (Annex 1)'!D69+'LCIA (Annex 1)'!D71+'LCIA (Annex 1)'!D73)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D66:D76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V130" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91))=0,0,('LCIA (Annex 1)'!D81+'LCIA (Annex 1)'!D84+'LCIA (Annex 1)'!D86+'LCIA (Annex 1)'!D88)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D81:D91)))</f>
+        <v>0.00552825552825553</v>
+      </c>
+      <c r="W130" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106))=0,0,('LCIA (Annex 1)'!D96+'LCIA (Annex 1)'!D99+'LCIA (Annex 1)'!D101+'LCIA (Annex 1)'!D103)/SUMPRODUCT(ABS('LCIA (Annex 1)'!D96:D106)))</f>
+        <v>0.000873007640977769</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P132" s="3" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P133" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q133" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="R133" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="S133" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="T133" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="U133" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="V133" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="W133" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P134" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q134" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16))=0,0,('LCIA (Annex 1)'!E14)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16)))</f>
+        <v>0.660670194003527</v>
+      </c>
+      <c r="R134" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31))=0,0,('LCIA (Annex 1)'!E29)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31)))</f>
+        <v>0.252109672963152</v>
+      </c>
+      <c r="S134" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46))=0,0,('LCIA (Annex 1)'!E44)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46)))</f>
+        <v>0.999919080757404</v>
+      </c>
+      <c r="T134" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61))=0,0,('LCIA (Annex 1)'!E59)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61)))</f>
+        <v>0.227272727272727</v>
+      </c>
+      <c r="U134" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76))=0,0,('LCIA (Annex 1)'!E74)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76)))</f>
+        <v>0.133333333333333</v>
+      </c>
+      <c r="V134" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91))=0,0,('LCIA (Annex 1)'!E89)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91)))</f>
+        <v>0.798064787547329</v>
+      </c>
+      <c r="W134" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106))=0,0,('LCIA (Annex 1)'!E104)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106)))</f>
+        <v>0.00011195871776734</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P135" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q135" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16))=0,0,('LCIA (Annex 1)'!E10)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16)))</f>
+        <v>0</v>
+      </c>
+      <c r="R135" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31))=0,0,('LCIA (Annex 1)'!E25)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31)))</f>
+        <v>0</v>
+      </c>
+      <c r="S135" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46))=0,0,('LCIA (Annex 1)'!E40)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T135" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61))=0,0,('LCIA (Annex 1)'!E55)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61)))</f>
+        <v>0.659090909090909</v>
+      </c>
+      <c r="U135" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76))=0,0,('LCIA (Annex 1)'!E70)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76)))</f>
+        <v>0.85</v>
+      </c>
+      <c r="V135" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91))=0,0,('LCIA (Annex 1)'!E85)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91)))</f>
+        <v>0</v>
+      </c>
+      <c r="W135" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106))=0,0,('LCIA (Annex 1)'!E100)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P136" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q136" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16))=0,0,('LCIA (Annex 1)'!E7)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16)))</f>
+        <v>0.167195767195767</v>
+      </c>
+      <c r="R136" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31))=0,0,('LCIA (Annex 1)'!E22)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31)))</f>
+        <v>0.65791765518484</v>
+      </c>
+      <c r="S136" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46))=0,0,('LCIA (Annex 1)'!E37)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T136" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61))=0,0,('LCIA (Annex 1)'!E52)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61)))</f>
+        <v>0.0681818181818182</v>
+      </c>
+      <c r="U136" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76))=0,0,('LCIA (Annex 1)'!E67)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76)))</f>
+        <v>0.0166666666666667</v>
+      </c>
+      <c r="V136" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91))=0,0,('LCIA (Annex 1)'!E82)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91)))</f>
+        <v>0.00504838031131679</v>
+      </c>
+      <c r="W136" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106))=0,0,('LCIA (Annex 1)'!E97)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106)))</f>
+        <v>0.00013740388089628</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P137" s="31" t="s">
+        <v>213</v>
+      </c>
+      <c r="Q137" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16))=0,0,('LCIA (Annex 1)'!E15)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16)))</f>
+        <v>0.1336860670194</v>
+      </c>
+      <c r="R137" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31))=0,0,('LCIA (Annex 1)'!E30)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31)))</f>
+        <v>0.0641560807631861</v>
+      </c>
+      <c r="S137" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46))=0,0,('LCIA (Annex 1)'!E45)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T137" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61))=0,0,('LCIA (Annex 1)'!E60)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61)))</f>
+        <v>0.0454545454545455</v>
+      </c>
+      <c r="U137" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76))=0,0,('LCIA (Annex 1)'!E75)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V137" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91))=0,0,('LCIA (Annex 1)'!E90)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91)))</f>
+        <v>0.00210349179638199</v>
+      </c>
+      <c r="W137" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106))=0,0,('LCIA (Annex 1)'!E105)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106)))</f>
+        <v>7.63354893868225E-006</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P138" s="31" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q138" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16))=0,0,('LCIA (Annex 1)'!E12)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16)))</f>
+        <v>0.00529100529100529</v>
+      </c>
+      <c r="R138" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31))=0,0,('LCIA (Annex 1)'!E27)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31)))</f>
+        <v>0.00555572239406589</v>
+      </c>
+      <c r="S138" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46))=0,0,('LCIA (Annex 1)'!E42)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T138" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61))=0,0,('LCIA (Annex 1)'!E57)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U138" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76))=0,0,('LCIA (Annex 1)'!E72)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V138" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91))=0,0,('LCIA (Annex 1)'!E87)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91)))</f>
+        <v>0</v>
+      </c>
+      <c r="W138" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106))=0,0,('LCIA (Annex 1)'!E102)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P139" s="31" t="s">
+        <v>239</v>
+      </c>
+      <c r="Q139" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16))=0,0,('LCIA (Annex 1)'!E16)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16)))</f>
+        <v>0</v>
+      </c>
+      <c r="R139" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31))=0,0,('LCIA (Annex 1)'!E31)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31)))</f>
+        <v>0</v>
+      </c>
+      <c r="S139" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46))=0,0,('LCIA (Annex 1)'!E46)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T139" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61))=0,0,('LCIA (Annex 1)'!E61)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U139" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76))=0,0,('LCIA (Annex 1)'!E76)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V139" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91))=0,0,('LCIA (Annex 1)'!E91)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91)))</f>
+        <v>0.193521245267143</v>
+      </c>
+      <c r="W139" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106))=0,0,('LCIA (Annex 1)'!E106)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106)))</f>
+        <v>0.501440196233098</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P140" s="31" t="s">
+        <v>206</v>
+      </c>
+      <c r="Q140" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16))=0,0,('LCIA (Annex 1)'!E8)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16)))</f>
+        <v>0</v>
+      </c>
+      <c r="R140" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31))=0,0,('LCIA (Annex 1)'!E23)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31)))</f>
+        <v>0</v>
+      </c>
+      <c r="S140" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46))=0,0,('LCIA (Annex 1)'!E38)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46)))</f>
+        <v>0</v>
+      </c>
+      <c r="T140" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61))=0,0,('LCIA (Annex 1)'!E53)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U140" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76))=0,0,('LCIA (Annex 1)'!E68)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V140" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91))=0,0,('LCIA (Annex 1)'!E83)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91)))</f>
+        <v>0</v>
+      </c>
+      <c r="W140" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106))=0,0,('LCIA (Annex 1)'!E98)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106)))</f>
+        <v>0.498290085037735</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P141" s="31" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q141" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16))=0,0,('LCIA (Annex 1)'!E6+'LCIA (Annex 1)'!E9+'LCIA (Annex 1)'!E11+'LCIA (Annex 1)'!E13)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E6:E16)))</f>
+        <v>0.0331569664902998</v>
+      </c>
+      <c r="R141" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31))=0,0,('LCIA (Annex 1)'!E21+'LCIA (Annex 1)'!E24+'LCIA (Annex 1)'!E26+'LCIA (Annex 1)'!E28)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E21:E31)))</f>
+        <v>0.0202608686947556</v>
+      </c>
+      <c r="S141" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46))=0,0,('LCIA (Annex 1)'!E36+'LCIA (Annex 1)'!E39+'LCIA (Annex 1)'!E41+'LCIA (Annex 1)'!E43)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E36:E46)))</f>
+        <v>8.09192425958893E-005</v>
+      </c>
+      <c r="T141" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61))=0,0,('LCIA (Annex 1)'!E51+'LCIA (Annex 1)'!E54+'LCIA (Annex 1)'!E56+'LCIA (Annex 1)'!E58)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E51:E61)))</f>
+        <v>0</v>
+      </c>
+      <c r="U141" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76))=0,0,('LCIA (Annex 1)'!E66+'LCIA (Annex 1)'!E69+'LCIA (Annex 1)'!E71+'LCIA (Annex 1)'!E73)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E66:E76)))</f>
+        <v>0</v>
+      </c>
+      <c r="V141" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91))=0,0,('LCIA (Annex 1)'!E81+'LCIA (Annex 1)'!E84+'LCIA (Annex 1)'!E86+'LCIA (Annex 1)'!E88)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E81:E91)))</f>
+        <v>0.0012620950778292</v>
+      </c>
+      <c r="W141" s="23" t="n">
+        <f aca="false">IF(SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106))=0,0,('LCIA (Annex 1)'!E96+'LCIA (Annex 1)'!E99+'LCIA (Annex 1)'!E101+'LCIA (Annex 1)'!E103)/SUMPRODUCT(ABS('LCIA (Annex 1)'!E96:E106)))</f>
+        <v>1.27225815644704E-005</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="2" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P147" s="3" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P148" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="Q148" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="R148" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="S148" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="T148" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="U148" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="V148" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="W148" s="5" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P149" s="31" t="s">
+        <v>393</v>
+      </c>
+      <c r="Q149" s="14" t="n">
+        <f aca="false">'KPI framework'!F8</f>
+        <v>2552.4</v>
+      </c>
+      <c r="R149" s="14" t="n">
+        <f aca="false">'KPI framework'!G8</f>
+        <v>2801</v>
+      </c>
+      <c r="S149" s="14" t="n">
+        <f aca="false">'KPI framework'!H8</f>
+        <v>1255</v>
+      </c>
+      <c r="T149" s="14" t="n">
+        <f aca="false">'KPI framework'!I8</f>
+        <v>2836</v>
+      </c>
+      <c r="U149" s="14" t="str">
+        <f aca="false">'KPI framework'!J8</f>
+        <v>✗</v>
+      </c>
+      <c r="V149" s="14" t="str">
+        <f aca="false">'KPI framework'!K8</f>
+        <v>✓</v>
+      </c>
+      <c r="W149" s="14" t="str">
+        <f aca="false">'KPI framework'!L8</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P150" s="31" t="s">
+        <v>394</v>
+      </c>
+      <c r="Q150" s="14" t="n">
+        <f aca="false">'KPI framework'!F9</f>
+        <v>89907.3</v>
+      </c>
+      <c r="R150" s="14" t="n">
+        <f aca="false">'KPI framework'!G9</f>
+        <v>90127</v>
+      </c>
+      <c r="S150" s="14" t="n">
+        <f aca="false">'KPI framework'!H9</f>
+        <v>19097</v>
+      </c>
+      <c r="T150" s="14" t="n">
+        <f aca="false">'KPI framework'!I9</f>
+        <v>99897</v>
+      </c>
+      <c r="U150" s="14" t="str">
+        <f aca="false">'KPI framework'!J9</f>
+        <v>✗</v>
+      </c>
+      <c r="V150" s="14" t="str">
+        <f aca="false">'KPI framework'!K9</f>
+        <v>✓</v>
+      </c>
+      <c r="W150" s="14" t="str">
+        <f aca="false">'KPI framework'!L9</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P151" s="31" t="s">
+        <v>395</v>
+      </c>
+      <c r="Q151" s="14" t="n">
+        <f aca="false">'KPI framework'!F10</f>
+        <v>11122.2</v>
+      </c>
+      <c r="R151" s="14" t="n">
+        <f aca="false">'KPI framework'!G10</f>
+        <v>10478</v>
+      </c>
+      <c r="S151" s="14" t="n">
+        <f aca="false">'KPI framework'!H10</f>
+        <v>4402</v>
+      </c>
+      <c r="T151" s="14" t="n">
+        <f aca="false">'KPI framework'!I10</f>
+        <v>12358</v>
+      </c>
+      <c r="U151" s="14" t="str">
+        <f aca="false">'KPI framework'!J10</f>
+        <v>✓</v>
+      </c>
+      <c r="V151" s="14" t="str">
+        <f aca="false">'KPI framework'!K10</f>
+        <v>✓</v>
+      </c>
+      <c r="W151" s="14" t="str">
+        <f aca="false">'KPI framework'!L10</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P152" s="31" t="s">
+        <v>396</v>
+      </c>
+      <c r="Q152" s="14" t="n">
+        <f aca="false">'KPI framework'!F11</f>
+        <v>40.5</v>
+      </c>
+      <c r="R152" s="14" t="n">
+        <f aca="false">'KPI framework'!G11</f>
+        <v>42</v>
+      </c>
+      <c r="S152" s="14" t="n">
+        <f aca="false">'KPI framework'!H11</f>
+        <v>6</v>
+      </c>
+      <c r="T152" s="14" t="n">
+        <f aca="false">'KPI framework'!I11</f>
+        <v>45</v>
+      </c>
+      <c r="U152" s="14" t="str">
+        <f aca="false">'KPI framework'!J11</f>
+        <v>✗</v>
+      </c>
+      <c r="V152" s="14" t="str">
+        <f aca="false">'KPI framework'!K11</f>
+        <v>✓</v>
+      </c>
+      <c r="W152" s="14" t="str">
+        <f aca="false">'KPI framework'!L11</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P153" s="31" t="s">
+        <v>397</v>
+      </c>
+      <c r="Q153" s="14" t="n">
+        <f aca="false">'KPI framework'!F12</f>
+        <v>54.9</v>
+      </c>
+      <c r="R153" s="14" t="n">
+        <f aca="false">'KPI framework'!G12</f>
+        <v>26</v>
+      </c>
+      <c r="S153" s="14" t="n">
+        <f aca="false">'KPI framework'!H12</f>
+        <v>2</v>
+      </c>
+      <c r="T153" s="14" t="n">
+        <f aca="false">'KPI framework'!I12</f>
+        <v>61</v>
+      </c>
+      <c r="U153" s="14" t="str">
+        <f aca="false">'KPI framework'!J12</f>
+        <v>✓</v>
+      </c>
+      <c r="V153" s="14" t="str">
+        <f aca="false">'KPI framework'!K12</f>
+        <v>✓</v>
+      </c>
+      <c r="W153" s="14" t="str">
+        <f aca="false">'KPI framework'!L12</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P154" s="31" t="s">
+        <v>398</v>
+      </c>
+      <c r="Q154" s="14" t="n">
+        <f aca="false">'KPI framework'!F13</f>
+        <v>2141.1</v>
+      </c>
+      <c r="R154" s="14" t="n">
+        <f aca="false">'KPI framework'!G13</f>
+        <v>2946</v>
+      </c>
+      <c r="S154" s="14" t="n">
+        <f aca="false">'KPI framework'!H13</f>
+        <v>4885</v>
+      </c>
+      <c r="T154" s="14" t="n">
+        <f aca="false">'KPI framework'!I13</f>
+        <v>2379</v>
+      </c>
+      <c r="U154" s="14" t="str">
+        <f aca="false">'KPI framework'!J13</f>
+        <v>✗</v>
+      </c>
+      <c r="V154" s="14" t="str">
+        <f aca="false">'KPI framework'!K13</f>
+        <v>✗</v>
+      </c>
+      <c r="W154" s="14" t="str">
+        <f aca="false">'KPI framework'!L13</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P155" s="31" t="s">
+        <v>399</v>
+      </c>
+      <c r="Q155" s="14" t="n">
+        <f aca="false">'KPI framework'!F14</f>
+        <v>353701.8</v>
+      </c>
+      <c r="R155" s="14" t="n">
+        <f aca="false">'KPI framework'!G14</f>
+        <v>163840</v>
+      </c>
+      <c r="S155" s="14" t="n">
+        <f aca="false">'KPI framework'!H14</f>
+        <v>115691</v>
+      </c>
+      <c r="T155" s="14" t="n">
+        <f aca="false">'KPI framework'!I14</f>
+        <v>393002</v>
+      </c>
+      <c r="U155" s="14" t="str">
+        <f aca="false">'KPI framework'!J14</f>
+        <v>✓</v>
+      </c>
+      <c r="V155" s="14" t="str">
+        <f aca="false">'KPI framework'!K14</f>
+        <v>✓</v>
+      </c>
+      <c r="W155" s="14" t="str">
+        <f aca="false">'KPI framework'!L14</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P156" s="31" t="s">
+        <v>400</v>
+      </c>
+      <c r="Q156" s="20" t="n">
+        <f aca="false">'KPI framework'!F15</f>
+        <v>0.35</v>
+      </c>
+      <c r="R156" s="20" t="n">
+        <f aca="false">'KPI framework'!G15</f>
+        <v>0.469758878127522</v>
+      </c>
+      <c r="S156" s="20" t="n">
+        <f aca="false">'KPI framework'!H15</f>
+        <v>1.1060393258427</v>
+      </c>
+      <c r="T156" s="20" t="n">
+        <f aca="false">'KPI framework'!I15</f>
+        <v>0.201757240481614</v>
+      </c>
+      <c r="U156" s="20" t="str">
+        <f aca="false">'KPI framework'!J15</f>
+        <v>✓</v>
+      </c>
+      <c r="V156" s="20" t="str">
+        <f aca="false">'KPI framework'!K15</f>
+        <v>✓</v>
+      </c>
+      <c r="W156" s="20" t="str">
+        <f aca="false">'KPI framework'!L15</f>
+        <v>✗</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P157" s="31" t="s">
+        <v>401</v>
+      </c>
+      <c r="Q157" s="20" t="n">
+        <f aca="false">'KPI framework'!F16</f>
+        <v>0.3</v>
+      </c>
+      <c r="R157" s="20" t="n">
+        <f aca="false">'KPI framework'!G16</f>
+        <v>0.3215799031477</v>
+      </c>
+      <c r="S157" s="20" t="n">
+        <f aca="false">'KPI framework'!H16</f>
+        <v>0.950734658599827</v>
+      </c>
+      <c r="T157" s="20" t="n">
+        <f aca="false">'KPI framework'!I16</f>
+        <v>0.162707452001302</v>
+      </c>
+      <c r="U157" s="20" t="str">
+        <f aca="false">'KPI framework'!J16</f>
+        <v>✓</v>
+      </c>
+      <c r="V157" s="20" t="str">
+        <f aca="false">'KPI framework'!K16</f>
+        <v>✓</v>
+      </c>
+      <c r="W157" s="20" t="str">
+        <f aca="false">'KPI framework'!L16</f>
+        <v>✗</v>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P158" s="31" t="s">
+        <v>402</v>
+      </c>
+      <c r="Q158" s="14" t="n">
+        <f aca="false">'KPI framework'!F17</f>
+        <v>60</v>
+      </c>
+      <c r="R158" s="14" t="n">
+        <f aca="false">'KPI framework'!G17</f>
+        <v>54.7384865744508</v>
+      </c>
+      <c r="S158" s="14" t="n">
+        <f aca="false">'KPI framework'!H17</f>
+        <v>-3.79874213836478</v>
+      </c>
+      <c r="T158" s="14" t="n">
+        <f aca="false">'KPI framework'!I17</f>
+        <v>95.9296072999837</v>
+      </c>
+      <c r="U158" s="14" t="str">
+        <f aca="false">'KPI framework'!J17</f>
+        <v>✓</v>
+      </c>
+      <c r="V158" s="14" t="str">
+        <f aca="false">'KPI framework'!K17</f>
+        <v>✓</v>
+      </c>
+      <c r="W158" s="14" t="str">
+        <f aca="false">'KPI framework'!L17</f>
+        <v>✗</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P159" s="31" t="s">
+        <v>403</v>
+      </c>
+      <c r="Q159" s="14" t="n">
+        <f aca="false">'KPI framework'!F18</f>
+        <v>1.75</v>
+      </c>
+      <c r="R159" s="14" t="n">
+        <f aca="false">'KPI framework'!G18</f>
+        <v>1.7179253867152</v>
+      </c>
+      <c r="S159" s="14" t="n">
+        <f aca="false">'KPI framework'!H18</f>
+        <v>1.36923076923077</v>
+      </c>
+      <c r="T159" s="14" t="n">
+        <f aca="false">'KPI framework'!I18</f>
+        <v>1.78833306175656</v>
+      </c>
+      <c r="U159" s="14" t="str">
+        <f aca="false">'KPI framework'!J18</f>
+        <v>✓</v>
+      </c>
+      <c r="V159" s="14" t="str">
+        <f aca="false">'KPI framework'!K18</f>
+        <v>✓</v>
+      </c>
+      <c r="W159" s="14" t="str">
+        <f aca="false">'KPI framework'!L18</f>
+        <v>✗</v>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P160" s="31" t="s">
+        <v>404</v>
+      </c>
+      <c r="Q160" s="20" t="n">
+        <f aca="false">'KPI framework'!F19</f>
+        <v>0.5</v>
+      </c>
+      <c r="R160" s="20" t="n">
+        <f aca="false">'KPI framework'!G19</f>
+        <v>0.551977170811252</v>
+      </c>
+      <c r="S160" s="20" t="n">
+        <f aca="false">'KPI framework'!H19</f>
+        <v>0.998172052082455</v>
+      </c>
+      <c r="T160" s="20" t="n">
+        <f aca="false">'KPI framework'!I19</f>
+        <v>0</v>
+      </c>
+      <c r="U160" s="20" t="str">
+        <f aca="false">'KPI framework'!J19</f>
+        <v>✓</v>
+      </c>
+      <c r="V160" s="20" t="str">
+        <f aca="false">'KPI framework'!K19</f>
+        <v>✓</v>
+      </c>
+      <c r="W160" s="20" t="str">
+        <f aca="false">'KPI framework'!L19</f>
+        <v>✗</v>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P161" s="31" t="s">
+        <v>405</v>
+      </c>
+      <c r="Q161" s="20" t="n">
+        <f aca="false">'KPI framework'!F20</f>
+        <v>0.6</v>
+      </c>
+      <c r="R161" s="20" t="n">
+        <f aca="false">'KPI framework'!G20</f>
+        <v>0.553016779721528</v>
+      </c>
+      <c r="S161" s="20" t="n">
+        <f aca="false">'KPI framework'!H20</f>
+        <v>0.58406374501992</v>
+      </c>
+      <c r="T161" s="20" t="n">
+        <f aca="false">'KPI framework'!I20</f>
+        <v>0.660437235543018</v>
+      </c>
+      <c r="U161" s="20" t="str">
+        <f aca="false">'KPI framework'!J20</f>
+        <v>✓</v>
+      </c>
+      <c r="V161" s="20" t="str">
+        <f aca="false">'KPI framework'!K20</f>
+        <v>✓</v>
+      </c>
+      <c r="W161" s="20" t="str">
+        <f aca="false">'KPI framework'!L20</f>
+        <v>✗</v>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P162" s="31" t="s">
+        <v>330</v>
+      </c>
+      <c r="Q162" s="12"/>
+      <c r="R162" s="12"/>
+      <c r="S162" s="12"/>
+      <c r="T162" s="12"/>
+      <c r="U162" s="12" t="str">
+        <f aca="false">'KPI framework'!J22</f>
+        <v>9 / 13</v>
+      </c>
+      <c r="V162" s="12" t="str">
+        <f aca="false">'KPI framework'!K22</f>
+        <v>12 / 13</v>
+      </c>
+      <c r="W162" s="12" t="str">
+        <f aca="false">'KPI framework'!L22</f>
+        <v>0 / 13</v>
+      </c>
+    </row>
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="2" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P182" s="3" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="183" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P183" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="Q183" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="R183" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="S183" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P184" s="31" t="s">
+        <v>286</v>
+      </c>
+      <c r="Q184" s="23" t="n">
+        <f aca="false">Comparison!C5/Comparison!$E5</f>
+        <v>0.987658674188999</v>
+      </c>
+      <c r="R184" s="23" t="n">
+        <f aca="false">Comparison!D5/Comparison!$E5</f>
+        <v>0.442524682651622</v>
+      </c>
+      <c r="S184" s="23" t="n">
+        <f aca="false">Comparison!E5/Comparison!$E5</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P185" s="31" t="s">
+        <v>292</v>
+      </c>
+      <c r="Q185" s="23" t="n">
+        <f aca="false">Comparison!C6/Comparison!$E6</f>
+        <v>0.902199265243201</v>
+      </c>
+      <c r="R185" s="23" t="n">
+        <f aca="false">Comparison!D6/Comparison!$E6</f>
+        <v>0.191166901908966</v>
+      </c>
+      <c r="S185" s="23" t="n">
+        <f aca="false">Comparison!E6/Comparison!$E6</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P186" s="31" t="s">
+        <v>295</v>
+      </c>
+      <c r="Q186" s="23" t="n">
+        <f aca="false">Comparison!C7/Comparison!$E7</f>
+        <v>0.847871823919728</v>
+      </c>
+      <c r="R186" s="23" t="n">
+        <f aca="false">Comparison!D7/Comparison!$E7</f>
+        <v>0.356206505907105</v>
+      </c>
+      <c r="S186" s="23" t="n">
+        <f aca="false">Comparison!E7/Comparison!$E7</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P187" s="31" t="s">
+        <v>298</v>
+      </c>
+      <c r="Q187" s="23" t="n">
+        <f aca="false">Comparison!C8/Comparison!$E8</f>
+        <v>0.933333333333333</v>
+      </c>
+      <c r="R187" s="23" t="n">
+        <f aca="false">Comparison!D8/Comparison!$E8</f>
+        <v>0.133333333333333</v>
+      </c>
+      <c r="S187" s="23" t="n">
+        <f aca="false">Comparison!E8/Comparison!$E8</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P188" s="31" t="s">
+        <v>301</v>
+      </c>
+      <c r="Q188" s="23" t="n">
+        <f aca="false">Comparison!C9/Comparison!$E9</f>
+        <v>0.426229508196721</v>
+      </c>
+      <c r="R188" s="23" t="n">
+        <f aca="false">Comparison!D9/Comparison!$E9</f>
+        <v>0.0327868852459016</v>
+      </c>
+      <c r="S188" s="23" t="n">
+        <f aca="false">Comparison!E9/Comparison!$E9</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P189" s="31" t="s">
+        <v>304</v>
+      </c>
+      <c r="Q189" s="23" t="n">
+        <f aca="false">Comparison!C10/Comparison!$E10</f>
+        <v>1.23833543505675</v>
+      </c>
+      <c r="R189" s="23" t="n">
+        <f aca="false">Comparison!D10/Comparison!$E10</f>
+        <v>2.05338377469525</v>
+      </c>
+      <c r="S189" s="23" t="n">
+        <f aca="false">Comparison!E10/Comparison!$E10</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P190" s="31" t="s">
+        <v>307</v>
+      </c>
+      <c r="Q190" s="23" t="n">
+        <f aca="false">Comparison!C11/Comparison!$E11</f>
+        <v>0.416893552704566</v>
+      </c>
+      <c r="R190" s="23" t="n">
+        <f aca="false">Comparison!D11/Comparison!$E11</f>
+        <v>0.294377636755029</v>
+      </c>
+      <c r="S190" s="23" t="n">
+        <f aca="false">Comparison!E11/Comparison!$E11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="2" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P223" s="3" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P224" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="Q224" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="R224" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="S224" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P225" s="31" t="s">
+        <v>411</v>
+      </c>
+      <c r="Q225" s="21" t="n">
+        <f aca="false">Inventory!C24</f>
+        <v>1229</v>
+      </c>
+      <c r="R225" s="21" t="n">
+        <f aca="false">Inventory!D24</f>
+        <v>159</v>
+      </c>
+      <c r="S225" s="21" t="n">
+        <f aca="false">Inventory!E24</f>
+        <v>6137</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P226" s="31" t="s">
+        <v>412</v>
+      </c>
+      <c r="Q226" s="39" t="n">
+        <f aca="false">Inventory!C25</f>
+        <v>0.813669650122051</v>
+      </c>
+      <c r="R226" s="39" t="n">
+        <f aca="false">Inventory!D25</f>
+        <v>6.28930817610063</v>
+      </c>
+      <c r="S226" s="39" t="n">
+        <f aca="false">Inventory!E25</f>
+        <v>0.162946064852534</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P227" s="31" t="s">
+        <v>413</v>
+      </c>
+      <c r="Q227" s="16" t="n">
+        <f aca="false">'Nutrient balance'!C8</f>
+        <v>126.8736</v>
+      </c>
+      <c r="R227" s="16" t="n">
+        <f aca="false">'Nutrient balance'!D8</f>
+        <v>5.696</v>
+      </c>
+      <c r="S227" s="16" t="n">
+        <f aca="false">'Nutrient balance'!E8</f>
+        <v>737.52</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A228" s="2" t="s">
-        <v>376</v>
+      <c r="P228" s="31" t="s">
+        <v>414</v>
+      </c>
+      <c r="Q228" s="23" t="n">
+        <f aca="false">'Nutrient balance'!C13</f>
+        <v>0.469758878127522</v>
+      </c>
+      <c r="R228" s="23" t="n">
+        <f aca="false">'Nutrient balance'!D13</f>
+        <v>1.1060393258427</v>
+      </c>
+      <c r="S228" s="23" t="n">
+        <f aca="false">'Nutrient balance'!E13</f>
+        <v>0.201757240481614</v>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P229" s="31" t="s">
+        <v>415</v>
+      </c>
+      <c r="Q229" s="23" t="n">
+        <f aca="false">'KPI framework'!$F$5</f>
+        <v>0.1</v>
+      </c>
+      <c r="R229" s="23" t="n">
+        <f aca="false">'KPI framework'!$F$5</f>
+        <v>0.1</v>
+      </c>
+      <c r="S229" s="23" t="n">
+        <f aca="false">'KPI framework'!$F$5</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P230" s="31" t="s">
+        <v>416</v>
+      </c>
+      <c r="Q230" s="12" t="str">
+        <f aca="false">'KPI framework'!J22</f>
+        <v>9 / 13</v>
+      </c>
+      <c r="R230" s="12" t="str">
+        <f aca="false">'KPI framework'!K22</f>
+        <v>12 / 13</v>
+      </c>
+      <c r="S230" s="12" t="str">
+        <f aca="false">'KPI framework'!L22</f>
+        <v>0 / 13</v>
+      </c>
+    </row>
+    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A244" s="2" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P245" s="3" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="246" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P246" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="Q246" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="R246" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="S246" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P247" s="31" t="s">
+        <v>354</v>
+      </c>
+      <c r="Q247" s="27" t="n">
+        <f aca="false">('KPI framework'!$F8-'KPI framework'!G8)/ABS('KPI framework'!$F8)</f>
+        <v>-0.0973985268766651</v>
+      </c>
+      <c r="R247" s="27" t="n">
+        <f aca="false">('KPI framework'!$F8-'KPI framework'!H8)/ABS('KPI framework'!$F8)</f>
+        <v>0.508305908164864</v>
+      </c>
+      <c r="S247" s="27" t="str">
+        <f aca="false">"baseline"</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P248" s="31" t="s">
+        <v>355</v>
+      </c>
+      <c r="Q248" s="27" t="n">
+        <f aca="false">('KPI framework'!$F9-'KPI framework'!G9)/ABS('KPI framework'!$F9)</f>
+        <v>-0.00244362804800052</v>
+      </c>
+      <c r="R248" s="27" t="n">
+        <f aca="false">('KPI framework'!$F9-'KPI framework'!H9)/ABS('KPI framework'!$F9)</f>
+        <v>0.78759233121226</v>
+      </c>
+      <c r="S248" s="27" t="str">
+        <f aca="false">"baseline"</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P249" s="31" t="s">
+        <v>356</v>
+      </c>
+      <c r="Q249" s="27" t="n">
+        <f aca="false">('KPI framework'!$F10-'KPI framework'!G10)/ABS('KPI framework'!$F10)</f>
+        <v>0.0579201956447466</v>
+      </c>
+      <c r="R249" s="27" t="n">
+        <f aca="false">('KPI framework'!$F10-'KPI framework'!H10)/ABS('KPI framework'!$F10)</f>
+        <v>0.60421499343655</v>
+      </c>
+      <c r="S249" s="27" t="str">
+        <f aca="false">"baseline"</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P250" s="31" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q250" s="27" t="n">
+        <f aca="false">('KPI framework'!$F11-'KPI framework'!G11)/ABS('KPI framework'!$F11)</f>
+        <v>-0.037037037037037</v>
+      </c>
+      <c r="R250" s="27" t="n">
+        <f aca="false">('KPI framework'!$F11-'KPI framework'!H11)/ABS('KPI framework'!$F11)</f>
+        <v>0.851851851851852</v>
+      </c>
+      <c r="S250" s="27" t="str">
+        <f aca="false">"baseline"</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P251" s="31" t="s">
+        <v>358</v>
+      </c>
+      <c r="Q251" s="27" t="n">
+        <f aca="false">('KPI framework'!$F12-'KPI framework'!G12)/ABS('KPI framework'!$F12)</f>
+        <v>0.526411657559199</v>
+      </c>
+      <c r="R251" s="27" t="n">
+        <f aca="false">('KPI framework'!$F12-'KPI framework'!H12)/ABS('KPI framework'!$F12)</f>
+        <v>0.963570127504554</v>
+      </c>
+      <c r="S251" s="27" t="str">
+        <f aca="false">"baseline"</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P252" s="31" t="s">
+        <v>359</v>
+      </c>
+      <c r="Q252" s="27" t="n">
+        <f aca="false">('KPI framework'!$F13-'KPI framework'!G13)/ABS('KPI framework'!$F13)</f>
+        <v>-0.375928261174163</v>
+      </c>
+      <c r="R252" s="27" t="n">
+        <f aca="false">('KPI framework'!$F13-'KPI framework'!H13)/ABS('KPI framework'!$F13)</f>
+        <v>-1.28153752743917</v>
+      </c>
+      <c r="S252" s="27" t="str">
+        <f aca="false">"baseline"</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P253" s="31" t="s">
+        <v>360</v>
+      </c>
+      <c r="Q253" s="27" t="n">
+        <f aca="false">('KPI framework'!$F14-'KPI framework'!G14)/ABS('KPI framework'!$F14)</f>
+        <v>0.536784941439371</v>
+      </c>
+      <c r="R253" s="27" t="n">
+        <f aca="false">('KPI framework'!$F14-'KPI framework'!H14)/ABS('KPI framework'!$F14)</f>
+        <v>0.672913736938856</v>
+      </c>
+      <c r="S253" s="27" t="str">
+        <f aca="false">"baseline"</f>
+        <v>baseline</v>
+      </c>
+    </row>
+    <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P254" s="31" t="s">
+        <v>361</v>
+      </c>
+      <c r="Q254" s="27" t="n">
+        <f aca="false">('KPI framework'!G15-'KPI framework'!$F15)/ABS('KPI framework'!$F15)</f>
+        <v>0.342168223221492</v>
+      </c>
+      <c r="R254" s="27" t="n">
+        <f aca="false">('KPI framework'!H15-'KPI framework'!$F15)/ABS('KPI framework'!$F15)</f>
+        <v>2.16011235955056</v>
+      </c>
+      <c r="S254" s="27" t="n">
+        <f aca="false">('KPI framework'!I15-'KPI framework'!$F15)/ABS('KPI framework'!$F15)</f>
+        <v>-0.423550741481103</v>
+      </c>
+    </row>
+    <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P255" s="31" t="s">
+        <v>362</v>
+      </c>
+      <c r="Q255" s="27" t="n">
+        <f aca="false">('KPI framework'!G16-'KPI framework'!$F16)/ABS('KPI framework'!$F16)</f>
+        <v>0.0719330104923327</v>
+      </c>
+      <c r="R255" s="27" t="n">
+        <f aca="false">('KPI framework'!H16-'KPI framework'!$F16)/ABS('KPI framework'!$F16)</f>
+        <v>2.16911552866609</v>
+      </c>
+      <c r="S255" s="27" t="n">
+        <f aca="false">('KPI framework'!I16-'KPI framework'!$F16)/ABS('KPI framework'!$F16)</f>
+        <v>-0.457641826662328</v>
+      </c>
+    </row>
+    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P256" s="31" t="s">
+        <v>363</v>
+      </c>
+      <c r="Q256" s="27" t="n">
+        <f aca="false">('KPI framework'!$F17-'KPI framework'!G17)/ABS('KPI framework'!$F17)</f>
+        <v>0.0876918904258202</v>
+      </c>
+      <c r="R256" s="27" t="n">
+        <f aca="false">('KPI framework'!$F17-'KPI framework'!H17)/ABS('KPI framework'!$F17)</f>
+        <v>1.06331236897275</v>
+      </c>
+      <c r="S256" s="27" t="n">
+        <f aca="false">('KPI framework'!$F17-'KPI framework'!I17)/ABS('KPI framework'!$F17)</f>
+        <v>-0.598826788333062</v>
+      </c>
+    </row>
+    <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P257" s="31" t="s">
+        <v>364</v>
+      </c>
+      <c r="Q257" s="27" t="n">
+        <f aca="false">('KPI framework'!$F18-'KPI framework'!G18)/ABS('KPI framework'!$F18)</f>
+        <v>0.0183283504484597</v>
+      </c>
+      <c r="R257" s="27" t="n">
+        <f aca="false">('KPI framework'!$F18-'KPI framework'!H18)/ABS('KPI framework'!$F18)</f>
+        <v>0.217582417582418</v>
+      </c>
+      <c r="S257" s="27" t="n">
+        <f aca="false">('KPI framework'!$F18-'KPI framework'!I18)/ABS('KPI framework'!$F18)</f>
+        <v>-0.0219046067180334</v>
+      </c>
+    </row>
+    <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P258" s="31" t="s">
+        <v>365</v>
+      </c>
+      <c r="Q258" s="27" t="n">
+        <f aca="false">('KPI framework'!G19-'KPI framework'!$F19)/ABS('KPI framework'!$F19)</f>
+        <v>0.103954341622503</v>
+      </c>
+      <c r="R258" s="27" t="n">
+        <f aca="false">('KPI framework'!H19-'KPI framework'!$F19)/ABS('KPI framework'!$F19)</f>
+        <v>0.996344104164909</v>
+      </c>
+      <c r="S258" s="27" t="n">
+        <f aca="false">('KPI framework'!I19-'KPI framework'!$F19)/ABS('KPI framework'!$F19)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="P259" s="31" t="s">
+        <v>366</v>
+      </c>
+      <c r="Q259" s="27" t="n">
+        <f aca="false">('KPI framework'!$F20-'KPI framework'!G20)/ABS('KPI framework'!$F20)</f>
+        <v>0.0783053671307865</v>
+      </c>
+      <c r="R259" s="27" t="n">
+        <f aca="false">('KPI framework'!$F20-'KPI framework'!H20)/ABS('KPI framework'!$F20)</f>
+        <v>0.0265604249667994</v>
+      </c>
+      <c r="S259" s="27" t="n">
+        <f aca="false">('KPI framework'!$F20-'KPI framework'!I20)/ABS('KPI framework'!$F20)</f>
+        <v>-0.100728725905031</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="Q112:W119">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <color rgb="FF0F6E56"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q123:W130">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <color rgb="FF0F6E56"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q134:W141">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <color rgb="FF0F6E56"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -19943,7 +22482,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>377</v>
+        <v>419</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19953,33 +22492,33 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>378</v>
+        <v>420</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>344</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>379</v>
+        <v>421</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>380</v>
+        <v>422</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>381</v>
+        <v>423</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>382</v>
+        <v>424</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>383</v>
+        <v>425</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>384</v>
+        <v>426</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>385</v>
+        <v>427</v>
       </c>
       <c r="C5" s="34" t="n">
         <v>126.9</v>
@@ -19997,15 +22536,15 @@
         <v>✓</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>386</v>
+        <v>428</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>387</v>
+        <v>429</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>385</v>
+        <v>427</v>
       </c>
       <c r="C6" s="14" t="n">
         <f aca="false">'Nutrient balance'!C12</f>
@@ -20024,15 +22563,15 @@
         <v>✓</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>388</v>
+        <v>430</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>389</v>
+        <v>431</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>385</v>
+        <v>427</v>
       </c>
       <c r="C7" s="14" t="n">
         <f aca="false">'LCIA (Annex 1)'!C98</f>
@@ -20051,15 +22590,15 @@
         <v>✓</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>390</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>391</v>
+        <v>433</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>385</v>
+        <v>427</v>
       </c>
       <c r="C8" s="14" t="n">
         <f aca="false">Inventory!C21</f>
@@ -20078,15 +22617,15 @@
         <v>✓</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>392</v>
+        <v>434</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>393</v>
+        <v>435</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>385</v>
+        <v>427</v>
       </c>
       <c r="C9" s="14" t="n">
         <f aca="false">'LCIA (Annex 1)'!C91</f>
@@ -20105,15 +22644,15 @@
         <v>✓</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>394</v>
+        <v>436</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>384</v>
+        <v>426</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>395</v>
+        <v>437</v>
       </c>
       <c r="C10" s="34" t="n">
         <v>5.7</v>
@@ -20131,15 +22670,15 @@
         <v>✓</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>386</v>
+        <v>428</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>387</v>
+        <v>429</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>395</v>
+        <v>437</v>
       </c>
       <c r="C11" s="14" t="n">
         <f aca="false">'Nutrient balance'!D12</f>
@@ -20158,15 +22697,15 @@
         <v>✓</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>388</v>
+        <v>430</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>389</v>
+        <v>431</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>395</v>
+        <v>437</v>
       </c>
       <c r="C12" s="14" t="n">
         <f aca="false">'LCIA (Annex 1)'!D98</f>
@@ -20185,15 +22724,15 @@
         <v>✓</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>390</v>
+        <v>432</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>391</v>
+        <v>433</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>395</v>
+        <v>437</v>
       </c>
       <c r="C13" s="14" t="n">
         <f aca="false">Inventory!D21</f>
@@ -20212,15 +22751,15 @@
         <v>check</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>396</v>
+        <v>438</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>393</v>
+        <v>435</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>395</v>
+        <v>437</v>
       </c>
       <c r="C14" s="14" t="n">
         <f aca="false">'LCIA (Annex 1)'!D91</f>
@@ -20239,15 +22778,15 @@
         <v>✓</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>394</v>
+        <v>436</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>384</v>
+        <v>426</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>397</v>
+        <v>439</v>
       </c>
       <c r="C15" s="34" t="n">
         <v>737.5</v>
@@ -20265,15 +22804,15 @@
         <v>✓</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>386</v>
+        <v>428</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>387</v>
+        <v>429</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>397</v>
+        <v>439</v>
       </c>
       <c r="C16" s="14" t="n">
         <f aca="false">'Nutrient balance'!E12</f>
@@ -20292,15 +22831,15 @@
         <v>✓</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>388</v>
+        <v>430</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>389</v>
+        <v>431</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>397</v>
+        <v>439</v>
       </c>
       <c r="C17" s="14" t="n">
         <f aca="false">'LCIA (Annex 1)'!E98</f>
@@ -20319,15 +22858,15 @@
         <v>✓</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>390</v>
+        <v>432</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>391</v>
+        <v>433</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>397</v>
+        <v>439</v>
       </c>
       <c r="C18" s="14" t="n">
         <f aca="false">Inventory!E21</f>
@@ -20346,15 +22885,15 @@
         <v>✓</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>392</v>
+        <v>434</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>393</v>
+        <v>435</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>397</v>
+        <v>439</v>
       </c>
       <c r="C19" s="14" t="n">
         <f aca="false">'LCIA (Annex 1)'!E91</f>
@@ -20373,7 +22912,7 @@
         <v>check</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>398</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>
@@ -20409,7 +22948,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>399</v>
+        <v>441</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20419,58 +22958,58 @@
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="B4" s="39" t="s">
-        <v>401</v>
+        <v>442</v>
+      </c>
+      <c r="B4" s="40" t="s">
+        <v>443</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>402</v>
-      </c>
-      <c r="B5" s="39" t="s">
-        <v>403</v>
+        <v>444</v>
+      </c>
+      <c r="B5" s="40" t="s">
+        <v>445</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="39" t="s">
-        <v>404</v>
+      <c r="B6" s="40" t="s">
+        <v>446</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="B7" s="39" t="s">
-        <v>406</v>
+        <v>447</v>
+      </c>
+      <c r="B7" s="40" t="s">
+        <v>448</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="39" t="s">
-        <v>407</v>
+      <c r="B8" s="40" t="s">
+        <v>449</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="B9" s="39" t="s">
-        <v>409</v>
+        <v>450</v>
+      </c>
+      <c r="B9" s="40" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="B10" s="39" t="s">
-        <v>411</v>
+        <v>452</v>
+      </c>
+      <c r="B10" s="40" t="s">
+        <v>453</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove the repeated flow diagram pictures from the Excel tool
The Flow diagrams tab keeps the cell-drawn diagram and data table for
each system; the duplicate picture below each one is gone, and so is
the cairosvg dependency.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LS2wYESwFTwwPUQtk712Bb
</commit_message>
<xml_diff>
--- a/excel/IMTA_KPI_decision_tool.xlsx
+++ b/excel/IMTA_KPI_decision_tool.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1423" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1420" uniqueCount="570">
   <si>
     <t xml:space="preserve">Pond IMTA vs fish polyculture: LCA results and circular KPI decision tool</t>
   </si>
@@ -157,93 +157,96 @@
     <t xml:space="preserve">How the fish waste is used in each system, with the flows</t>
   </si>
   <si>
+    <t xml:space="preserve">Diagrams + data (live)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metadata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dataset description in the LCIS2024 structure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inventory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table 4 of the report per pond and cycle (yellow), scaled to 1 t of product</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input + calculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nutrient balance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N and P from feed to fish + oysters, macroalgae and water (Table 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LCI per tonne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foreground inventory for one functional unit, grouped into inputs and outputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LCIA (Annex 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impacts per tonne for 11 processes and 7 categories, with shares</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contribution analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of each process in each impact (heatmap) and contribution charts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculation + charts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Totals side by side and change against the fish-only pond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculation + chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KPI framework</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 KPIs with targets and pass / fail; the improvement target is in F5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dashboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Score per system and two summary charts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Results + charts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Radar profile, change vs baseline, N and P fate, targets met, margin to target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charts (live)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Report figures from make_charts.py, each with its data table</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pictures + data</t>
   </si>
   <si>
-    <t xml:space="preserve">Metadata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset description in the LCIS2024 structure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inventory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table 4 of the report per pond and cycle (yellow), scaled to 1 t of product</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Input + calculation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nutrient balance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N and P from feed to fish + oysters, macroalgae and water (Table 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LCI per tonne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Foreground inventory for one functional unit, grouped into inputs and outputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LCIA (Annex 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impacts per tonne for 11 processes and 7 categories, with shares</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contribution analysis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Share of each process in each impact (heatmap) and contribution charts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculation + charts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comparison</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Totals side by side and change against the fish-only pond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculation + chart</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KPI framework</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13 KPIs with targets and pass / fail; the improvement target is in F5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dashboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Score per system and two summary charts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Results + charts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Radar profile, change vs baseline, N and P fate, targets met, margin to target</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charts (live)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Report figures from make_charts.py, each with its data table</t>
-  </si>
-  <si>
     <t xml:space="preserve">Data checks</t>
   </si>
   <si>
@@ -454,7 +457,7 @@
     <t xml:space="preserve">Flow diagrams - how the fish waste is used in each system (per pond and production cycle)</t>
   </si>
   <si>
-    <t xml:space="preserve">Each system: a live flow diagram drawn with cells (numbers update with the inputs), the data table on the right, and the same diagram as a picture below.</t>
+    <t xml:space="preserve">Each system: a flow diagram drawn with cells and its data table on the right. All numbers are live: they update when you change an input.</t>
   </si>
   <si>
     <t xml:space="preserve">Fish feed</t>
@@ -566,9 +569,6 @@
   </si>
   <si>
     <t xml:space="preserve">%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same diagram as a picture (make_flow.py, published values):</t>
   </si>
   <si>
     <t xml:space="preserve">Ulva + Gracilaria take up N, P</t>
@@ -4065,11 +4065,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="68108669"/>
-        <c:axId val="71227753"/>
+        <c:axId val="534267"/>
+        <c:axId val="17071410"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="68108669"/>
+        <c:axId val="534267"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4135,7 +4135,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71227753"/>
+        <c:crossAx val="17071410"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4143,7 +4143,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71227753"/>
+        <c:axId val="17071410"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4220,7 +4220,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68108669"/>
+        <c:crossAx val="534267"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5055,11 +5055,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="14603149"/>
-        <c:axId val="62482951"/>
+        <c:axId val="16745668"/>
+        <c:axId val="77798033"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="14603149"/>
+        <c:axId val="16745668"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5091,7 +5091,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62482951"/>
+        <c:crossAx val="77798033"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5099,7 +5099,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="62482951"/>
+        <c:axId val="77798033"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5175,7 +5175,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14603149"/>
+        <c:crossAx val="16745668"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5490,11 +5490,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="61881104"/>
-        <c:axId val="60136410"/>
+        <c:axId val="88934295"/>
+        <c:axId val="65848690"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="61881104"/>
+        <c:axId val="88934295"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5526,7 +5526,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60136410"/>
+        <c:crossAx val="65848690"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5534,7 +5534,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60136410"/>
+        <c:axId val="65848690"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5610,7 +5610,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61881104"/>
+        <c:crossAx val="88934295"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6429,11 +6429,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="60016764"/>
-        <c:axId val="99270729"/>
+        <c:axId val="46963261"/>
+        <c:axId val="32525648"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="60016764"/>
+        <c:axId val="46963261"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6465,7 +6465,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99270729"/>
+        <c:crossAx val="32525648"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6473,7 +6473,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="99270729"/>
+        <c:axId val="32525648"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6549,7 +6549,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60016764"/>
+        <c:crossAx val="46963261"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6738,11 +6738,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="96914247"/>
-        <c:axId val="58466272"/>
+        <c:axId val="74289908"/>
+        <c:axId val="41877173"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="96914247"/>
+        <c:axId val="74289908"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6774,7 +6774,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58466272"/>
+        <c:crossAx val="41877173"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6782,7 +6782,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58466272"/>
+        <c:axId val="41877173"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6858,7 +6858,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96914247"/>
+        <c:crossAx val="74289908"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7269,11 +7269,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50684838"/>
-        <c:axId val="4322994"/>
+        <c:axId val="17950757"/>
+        <c:axId val="8309368"/>
       </c:radarChart>
       <c:catAx>
-        <c:axId val="50684838"/>
+        <c:axId val="17950757"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -7302,7 +7302,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4322994"/>
+        <c:crossAx val="8309368"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7310,7 +7310,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="4322994"/>
+        <c:axId val="8309368"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="2.5"/>
@@ -7354,7 +7354,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50684838"/>
+        <c:crossAx val="17950757"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="0.5"/>
@@ -7674,11 +7674,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="44689796"/>
-        <c:axId val="14668580"/>
+        <c:axId val="76079506"/>
+        <c:axId val="80918200"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="44689796"/>
+        <c:axId val="76079506"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -7710,7 +7710,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14668580"/>
+        <c:crossAx val="80918200"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7718,7 +7718,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="14668580"/>
+        <c:axId val="80918200"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1.5"/>
@@ -7762,7 +7762,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44689796"/>
+        <c:crossAx val="76079506"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8119,11 +8119,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="43312232"/>
-        <c:axId val="95332962"/>
+        <c:axId val="1837903"/>
+        <c:axId val="31716291"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="43312232"/>
+        <c:axId val="1837903"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -8155,7 +8155,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95332962"/>
+        <c:crossAx val="31716291"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8163,7 +8163,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95332962"/>
+        <c:axId val="31716291"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8239,7 +8239,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43312232"/>
+        <c:crossAx val="1837903"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8596,11 +8596,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="59309803"/>
-        <c:axId val="75812655"/>
+        <c:axId val="68274788"/>
+        <c:axId val="68897771"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="59309803"/>
+        <c:axId val="68274788"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -8632,7 +8632,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75812655"/>
+        <c:crossAx val="68897771"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8640,7 +8640,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75812655"/>
+        <c:axId val="68897771"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8716,7 +8716,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59309803"/>
+        <c:crossAx val="68274788"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8987,11 +8987,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="81986934"/>
-        <c:axId val="60130496"/>
+        <c:axId val="96883955"/>
+        <c:axId val="54046183"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="81986934"/>
+        <c:axId val="96883955"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9023,7 +9023,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60130496"/>
+        <c:crossAx val="54046183"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9031,7 +9031,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60130496"/>
+        <c:axId val="54046183"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -9109,7 +9109,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81986934"/>
+        <c:crossAx val="96883955"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -9626,11 +9626,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="56557951"/>
-        <c:axId val="26338504"/>
+        <c:axId val="8981486"/>
+        <c:axId val="44550519"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="56557951"/>
+        <c:axId val="8981486"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -9662,7 +9662,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26338504"/>
+        <c:crossAx val="44550519"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9670,7 +9670,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="26338504"/>
+        <c:axId val="44550519"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1.5"/>
@@ -9714,7 +9714,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56557951"/>
+        <c:crossAx val="8981486"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -10805,11 +10805,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="63645779"/>
-        <c:axId val="41777672"/>
+        <c:axId val="70525939"/>
+        <c:axId val="2444354"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="63645779"/>
+        <c:axId val="70525939"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -10875,7 +10875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41777672"/>
+        <c:crossAx val="2444354"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10883,7 +10883,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="41777672"/>
+        <c:axId val="2444354"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -10960,7 +10960,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63645779"/>
+        <c:crossAx val="70525939"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -12051,11 +12051,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="62806259"/>
-        <c:axId val="29498986"/>
+        <c:axId val="21955248"/>
+        <c:axId val="12226392"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="62806259"/>
+        <c:axId val="21955248"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -12121,7 +12121,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29498986"/>
+        <c:crossAx val="12226392"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -12129,7 +12129,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="29498986"/>
+        <c:axId val="12226392"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -12206,7 +12206,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62806259"/>
+        <c:crossAx val="21955248"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13041,11 +13041,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="9443518"/>
-        <c:axId val="58214215"/>
+        <c:axId val="4074245"/>
+        <c:axId val="32974001"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="9443518"/>
+        <c:axId val="4074245"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13077,7 +13077,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58214215"/>
+        <c:crossAx val="32974001"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13085,7 +13085,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58214215"/>
+        <c:axId val="32974001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13161,7 +13161,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9443518"/>
+        <c:crossAx val="4074245"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13996,11 +13996,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="53027728"/>
-        <c:axId val="59595012"/>
+        <c:axId val="25848431"/>
+        <c:axId val="96592042"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="53027728"/>
+        <c:axId val="25848431"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14032,7 +14032,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59595012"/>
+        <c:crossAx val="96592042"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -14040,7 +14040,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59595012"/>
+        <c:axId val="96592042"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14116,7 +14116,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53027728"/>
+        <c:crossAx val="25848431"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -14951,11 +14951,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="30068659"/>
-        <c:axId val="86150336"/>
+        <c:axId val="48022836"/>
+        <c:axId val="29955123"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="30068659"/>
+        <c:axId val="48022836"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14987,7 +14987,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86150336"/>
+        <c:crossAx val="29955123"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -14995,7 +14995,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86150336"/>
+        <c:axId val="29955123"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -15071,7 +15071,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30068659"/>
+        <c:crossAx val="48022836"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -15906,11 +15906,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="44963886"/>
-        <c:axId val="47734263"/>
+        <c:axId val="88745609"/>
+        <c:axId val="45201133"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="44963886"/>
+        <c:axId val="88745609"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -15942,7 +15942,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47734263"/>
+        <c:crossAx val="45201133"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -15950,7 +15950,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="47734263"/>
+        <c:axId val="45201133"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16026,7 +16026,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44963886"/>
+        <c:crossAx val="88745609"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -16861,11 +16861,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="172438"/>
-        <c:axId val="76132808"/>
+        <c:axId val="24257415"/>
+        <c:axId val="44245167"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="172438"/>
+        <c:axId val="24257415"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16897,7 +16897,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76132808"/>
+        <c:crossAx val="44245167"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -16905,7 +16905,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="76132808"/>
+        <c:axId val="44245167"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16981,7 +16981,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="172438"/>
+        <c:crossAx val="24257415"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -17816,11 +17816,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="31474867"/>
-        <c:axId val="80044651"/>
+        <c:axId val="39386110"/>
+        <c:axId val="2284601"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="31474867"/>
+        <c:axId val="39386110"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -17852,7 +17852,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80044651"/>
+        <c:crossAx val="2284601"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -17860,7 +17860,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80044651"/>
+        <c:axId val="2284601"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -17936,7 +17936,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31474867"/>
+        <c:crossAx val="39386110"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -17992,122 +17992,6 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>146160</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>184680</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>79200</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="4800600"/>
-          <a:ext cx="8572320" cy="4505040"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>68</xdr:row>
-      <xdr:rowOff>131400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>184680</xdr:colOff>
-      <xdr:row>92</xdr:row>
-      <xdr:rowOff>64440</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="13982760"/>
-          <a:ext cx="8572320" cy="4505040"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>114</xdr:row>
-      <xdr:rowOff>117000</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>184680</xdr:colOff>
-      <xdr:row>138</xdr:row>
-      <xdr:rowOff>50040</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="23164920"/>
-          <a:ext cx="8572320" cy="4505040"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>5</xdr:row>
@@ -18121,7 +18005,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 1"/>
+        <xdr:cNvPr id="0" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18151,7 +18035,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 2"/>
+        <xdr:cNvPr id="1" name="Chart 2"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18181,7 +18065,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 3"/>
+        <xdr:cNvPr id="2" name="Chart 3"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18211,7 +18095,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Chart 4"/>
+        <xdr:cNvPr id="3" name="Chart 4"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18241,7 +18125,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="7" name="Chart 5"/>
+        <xdr:cNvPr id="4" name="Chart 5"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18271,7 +18155,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="8" name="Chart 6"/>
+        <xdr:cNvPr id="5" name="Chart 6"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18301,7 +18185,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="9" name="Chart 7"/>
+        <xdr:cNvPr id="6" name="Chart 7"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18331,7 +18215,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="10" name="Chart 8"/>
+        <xdr:cNvPr id="7" name="Chart 8"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18361,7 +18245,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="11" name="Chart 9"/>
+        <xdr:cNvPr id="8" name="Chart 9"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18391,7 +18275,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="12" name="Chart 10"/>
+        <xdr:cNvPr id="9" name="Chart 10"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18409,7 +18293,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -18426,7 +18310,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="13" name="Chart 1"/>
+        <xdr:cNvPr id="10" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18444,7 +18328,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -18461,7 +18345,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="14" name="Chart 1"/>
+        <xdr:cNvPr id="11" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18491,7 +18375,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="15" name="Chart 2"/>
+        <xdr:cNvPr id="12" name="Chart 2"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18509,7 +18393,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -18526,7 +18410,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="16" name="Chart 1"/>
+        <xdr:cNvPr id="13" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18556,7 +18440,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="17" name="Chart 2"/>
+        <xdr:cNvPr id="14" name="Chart 2"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18586,7 +18470,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="18" name="Chart 3"/>
+        <xdr:cNvPr id="15" name="Chart 3"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18616,7 +18500,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="19" name="Chart 4"/>
+        <xdr:cNvPr id="16" name="Chart 4"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18646,7 +18530,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="20" name="Chart 5"/>
+        <xdr:cNvPr id="17" name="Chart 5"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18676,7 +18560,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="21" name="Chart 6"/>
+        <xdr:cNvPr id="18" name="Chart 6"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -18694,7 +18578,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -18711,7 +18595,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="22" name="Image 1" descr="Picture"/>
+        <xdr:cNvPr id="19" name="Image 1" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -18748,7 +18632,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="23" name="Image 2" descr="Picture"/>
+        <xdr:cNvPr id="20" name="Image 2" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -18785,7 +18669,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="24" name="Image 3" descr="Picture"/>
+        <xdr:cNvPr id="21" name="Image 3" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -18822,7 +18706,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="25" name="Image 4" descr="Picture"/>
+        <xdr:cNvPr id="22" name="Image 4" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -18859,7 +18743,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="26" name="Image 5" descr="Picture"/>
+        <xdr:cNvPr id="23" name="Image 5" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -18896,7 +18780,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="27" name="Image 6" descr="Picture"/>
+        <xdr:cNvPr id="24" name="Image 6" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -18933,7 +18817,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="28" name="Image 7" descr="Picture"/>
+        <xdr:cNvPr id="25" name="Image 7" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -18970,7 +18854,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="29" name="Image 8" descr="Picture"/>
+        <xdr:cNvPr id="26" name="Image 8" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -19007,7 +18891,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="30" name="Image 9" descr="Picture"/>
+        <xdr:cNvPr id="27" name="Image 9" descr="Picture"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -19684,28 +19568,28 @@
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
       <c r="F43" s="21" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D44" s="14"/>
       <c r="E44" s="14"/>
       <c r="F44" s="21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="20" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D45" s="14"/>
       <c r="E45" s="14"/>
@@ -19715,7 +19599,7 @@
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C47" s="5"/>
       <c r="D47" s="5"/>
@@ -19727,7 +19611,7 @@
         <v>1888</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D49" s="23"/>
       <c r="E49" s="23"/>
@@ -19739,7 +19623,7 @@
         <v>3776</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D50" s="23"/>
       <c r="E50" s="23"/>
@@ -19747,10 +19631,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="25" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D51" s="23"/>
       <c r="E51" s="23"/>
@@ -19758,10 +19642,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="26" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C52" s="23" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D52" s="23"/>
       <c r="E52" s="23"/>
@@ -19769,7 +19653,7 @@
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5"/>
@@ -19778,10 +19662,10 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8"/>
@@ -19789,46 +19673,46 @@
     </row>
     <row r="57" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C57" s="27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E57" s="11"/>
       <c r="F57" s="11"/>
     </row>
     <row r="58" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C58" s="27" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E58" s="11"/>
       <c r="F58" s="11"/>
     </row>
     <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C59" s="27" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E59" s="11"/>
       <c r="F59" s="11"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C61" s="5"/>
       <c r="D61" s="5"/>
@@ -19837,10 +19721,10 @@
     </row>
     <row r="63" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D63" s="11"/>
       <c r="E63" s="11"/>
@@ -19848,10 +19732,10 @@
     </row>
     <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C64" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D64" s="11"/>
       <c r="E64" s="11"/>
@@ -19859,10 +19743,10 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C65" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D65" s="11"/>
       <c r="E65" s="11"/>
@@ -19870,10 +19754,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C66" s="11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D66" s="11"/>
       <c r="E66" s="11"/>
@@ -19881,10 +19765,10 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D67" s="11"/>
       <c r="E67" s="11"/>
@@ -19892,10 +19776,10 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D68" s="11"/>
       <c r="E68" s="11"/>
@@ -20001,7 +19885,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20009,7 +19893,7 @@
         <v>379</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>11</v>
@@ -20227,7 +20111,7 @@
         <v>389</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C11" s="39" t="n">
         <f aca="false">'LCIA (Annex 1)'!C108</f>
@@ -20271,7 +20155,7 @@
         <v>22</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>11</v>
@@ -20397,7 +20281,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20422,7 +20306,7 @@
         <v>402</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>403</v>
@@ -20792,7 +20676,7 @@
         <v>28</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E15" s="14" t="s">
         <v>439</v>
@@ -20839,7 +20723,7 @@
         <v>442</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>439</v>
@@ -20980,7 +20864,7 @@
         <v>452</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>439</v>
@@ -21027,7 +20911,7 @@
         <v>455</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>416</v>
@@ -21164,7 +21048,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21493,7 +21377,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22258,7 +22142,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22693,7 +22577,7 @@
     </row>
     <row r="86" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P86" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="Q86" s="8" t="s">
         <v>11</v>
@@ -22707,7 +22591,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P87" s="14" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="Q87" s="44" t="n">
         <f aca="false">'Nutrient balance'!C8*Inventory!C25</f>
@@ -24321,7 +24205,7 @@
     </row>
     <row r="224" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P224" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q224" s="8" t="s">
         <v>11</v>
@@ -24745,7 +24629,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25206,12 +25090,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="28" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25232,7 +25116,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="34" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B6" s="100" t="s">
         <v>563</v>
@@ -25248,7 +25132,7 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="34" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B8" s="100" t="s">
         <v>565</v>
@@ -25296,122 +25180,122 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="28" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -25430,7 +25314,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K115"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -25448,17 +25332,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="28" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25468,19 +25352,19 @@
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="31" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E7" s="32" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G7" s="32" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I7" s="34" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25489,71 +25373,71 @@
         <v>1,888 kg · 126.9 kg N</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E8" s="36" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G8" s="36" t="str">
         <f aca="false">TEXT(Inventory!C19,"#,##0")&amp;" kg"</f>
         <v>130 kg</v>
       </c>
       <c r="I8" s="37" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J8" s="37" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K8" s="37" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D9" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I9" s="38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J9" s="39" t="n">
         <f aca="false">Inventory!C6</f>
         <v>1888</v>
       </c>
       <c r="K9" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E10" s="42" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G10" s="43" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J10" s="44" t="n">
         <f aca="false">'Nutrient balance'!C8</f>
         <v>126.8736</v>
       </c>
       <c r="K10" s="38" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25562,63 +25446,63 @@
         <v>683 kg stocked</v>
       </c>
       <c r="C11" s="46" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G11" s="47" t="str">
         <f aca="false">TEXT(Inventory!C18,"#,##0")&amp;" kg gained"</f>
         <v>1,099 kg gained</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J11" s="39" t="n">
         <f aca="false">Inventory!C8+Inventory!C9</f>
         <v>682.5</v>
       </c>
       <c r="K11" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D12" s="33" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J12" s="39" t="n">
         <f aca="false">Inventory!C7</f>
         <v>101110</v>
       </c>
       <c r="K12" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="48" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E13" s="49" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G13" s="49" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J13" s="39" t="n">
         <f aca="false">Inventory!C18</f>
         <v>1099</v>
       </c>
       <c r="K13" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25627,66 +25511,66 @@
         <v>101,110 m3 · pumped</v>
       </c>
       <c r="E14" s="51" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G14" s="51" t="str">
         <f aca="false">TEXT(Inventory!C20,"#,##0")&amp;" kg · "&amp;TEXT('Nutrient balance'!C10,"0.0")&amp;" kg N"</f>
         <v>1,224 kg · 30.6 kg N</v>
       </c>
       <c r="I14" s="38" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J14" s="39" t="n">
         <f aca="false">Inventory!C19</f>
         <v>130</v>
       </c>
       <c r="K14" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E15" s="33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J15" s="39" t="n">
         <f aca="false">Inventory!C20</f>
         <v>1224</v>
       </c>
       <c r="K15" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="52" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E16" s="53" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G16" s="34" t="str">
         <f aca="false">"N in products: "&amp;TEXT('Nutrient balance'!C9+'Nutrient balance'!C10,"0.0")&amp;" kg N"</f>
         <v>N in products: 59.6 kg N</v>
       </c>
       <c r="I16" s="38" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J16" s="44" t="n">
         <f aca="false">'Nutrient balance'!C9</f>
         <v>29</v>
       </c>
       <c r="K16" s="38" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="54" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E17" s="55" t="str">
         <f aca="false">IF('Nutrient balance'!C12&lt;0,"net uptake "&amp;TEXT(-'Nutrient balance'!C12,"0.0")&amp;" kg N",TEXT('Nutrient balance'!C12,"0.0")&amp;" kg N released")</f>
@@ -25697,626 +25581,611 @@
         <v>N use efficiency: 47%</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J17" s="44" t="n">
         <f aca="false">'Nutrient balance'!C10</f>
         <v>30.6</v>
       </c>
       <c r="K17" s="38" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I18" s="38" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J18" s="56" t="n">
         <f aca="false">'Nutrient balance'!C9+'Nutrient balance'!C10</f>
         <v>59.6</v>
       </c>
       <c r="K18" s="38" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I19" s="38" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J19" s="44" t="n">
         <f aca="false">'Nutrient balance'!C12</f>
         <v>67.2</v>
       </c>
       <c r="K19" s="38" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I20" s="38" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J20" s="57" t="n">
         <f aca="false">'Nutrient balance'!C13</f>
         <v>0.469758878127522</v>
       </c>
       <c r="K20" s="38" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="29" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="58" t="s">
+    <row r="24" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="58" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="31" t="s">
-        <v>140</v>
-      </c>
-      <c r="E53" s="32" t="s">
+    <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="F53" s="33" t="s">
+      <c r="E26" s="32" t="s">
         <v>142</v>
       </c>
-      <c r="G53" s="32" t="s">
+      <c r="F26" s="33" t="s">
         <v>143</v>
       </c>
-      <c r="I53" s="34" t="s">
+      <c r="G26" s="32" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="54" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="35" t="str">
+      <c r="I26" s="34" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="35" t="str">
         <f aca="false">TEXT(Inventory!D6,"#,##0")&amp;" kg · "&amp;TEXT('Nutrient balance'!D8,"#,##0.0")&amp;" kg N"</f>
         <v>89 kg · 5.7 kg N</v>
       </c>
-      <c r="B54" s="33" t="s">
-        <v>145</v>
-      </c>
-      <c r="E54" s="36" t="s">
+      <c r="B27" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="G54" s="36" t="str">
+      <c r="E27" s="36" t="s">
+        <v>147</v>
+      </c>
+      <c r="G27" s="36" t="str">
         <f aca="false">TEXT(Inventory!D19,"#,##0")&amp;" kg"</f>
         <v>94 kg</v>
       </c>
-      <c r="I54" s="37" t="s">
-        <v>147</v>
-      </c>
-      <c r="J54" s="37" t="s">
+      <c r="I27" s="37" t="s">
         <v>148</v>
       </c>
-      <c r="K54" s="37" t="s">
+      <c r="J27" s="37" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="55" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D55" s="33" t="s">
+      <c r="K27" s="37" t="s">
         <v>150</v>
       </c>
-      <c r="I55" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="J55" s="39" t="n">
+    </row>
+    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D28" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="I28" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="J28" s="39" t="n">
         <f aca="false">Inventory!D6</f>
         <v>89</v>
       </c>
-      <c r="K55" s="38" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="40" t="s">
+      <c r="K28" s="38" t="s">
         <v>152</v>
       </c>
-      <c r="B56" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="C56" s="41" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="40" t="s">
         <v>153</v>
       </c>
-      <c r="D56" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="E56" s="42" t="s">
+      <c r="B29" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="C29" s="41" t="s">
         <v>154</v>
       </c>
-      <c r="F56" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="G56" s="43" t="s">
+      <c r="D29" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="E29" s="42" t="s">
         <v>155</v>
       </c>
-      <c r="I56" s="38" t="s">
+      <c r="F29" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="G29" s="43" t="s">
         <v>156</v>
       </c>
-      <c r="J56" s="44" t="n">
+      <c r="I29" s="38" t="s">
+        <v>157</v>
+      </c>
+      <c r="J29" s="44" t="n">
         <f aca="false">'Nutrient balance'!D8</f>
         <v>5.696</v>
       </c>
-      <c r="K56" s="38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="45" t="str">
+      <c r="K29" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="45" t="str">
         <f aca="false">TEXT(Inventory!D8+Inventory!D9,"#,##0")&amp;" kg stocked"</f>
         <v>59 kg stocked</v>
       </c>
-      <c r="C57" s="46" t="s">
-        <v>158</v>
-      </c>
-      <c r="G57" s="47" t="str">
+      <c r="C30" s="46" t="s">
+        <v>159</v>
+      </c>
+      <c r="G30" s="47" t="str">
         <f aca="false">TEXT(Inventory!D18,"#,##0")&amp;" kg gained"</f>
         <v>65 kg gained</v>
       </c>
-      <c r="I57" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="J57" s="39" t="n">
+      <c r="I30" s="38" t="s">
+        <v>160</v>
+      </c>
+      <c r="J30" s="39" t="n">
         <f aca="false">Inventory!D8+Inventory!D9</f>
         <v>59.4</v>
       </c>
-      <c r="K57" s="38" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D58" s="33" t="s">
-        <v>145</v>
-      </c>
-      <c r="I58" s="38" t="s">
-        <v>160</v>
-      </c>
-      <c r="J58" s="39" t="n">
+      <c r="K30" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D31" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="I31" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="J31" s="39" t="n">
         <f aca="false">Inventory!D7</f>
         <v>7185</v>
       </c>
-      <c r="K58" s="38" t="s">
+      <c r="K31" s="38" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="48" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="59" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="48" t="s">
-        <v>160</v>
-      </c>
-      <c r="B59" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="E59" s="49" t="s">
-        <v>162</v>
-      </c>
-      <c r="F59" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="G59" s="49" t="s">
+      <c r="B32" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="E32" s="49" t="s">
         <v>163</v>
       </c>
-      <c r="I59" s="38" t="s">
+      <c r="F32" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="G32" s="49" t="s">
         <v>164</v>
       </c>
-      <c r="J59" s="39" t="n">
+      <c r="I32" s="38" t="s">
+        <v>165</v>
+      </c>
+      <c r="J32" s="39" t="n">
         <f aca="false">Inventory!D18</f>
         <v>65</v>
       </c>
-      <c r="K59" s="38" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="50" t="str">
+      <c r="K32" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="50" t="str">
         <f aca="false">TEXT(Inventory!D7,"#,##0")&amp;" m3 · tidal"</f>
         <v>7,185 m3 · tidal</v>
       </c>
-      <c r="E60" s="51" t="s">
+      <c r="E33" s="51" t="s">
         <v>178</v>
       </c>
-      <c r="G60" s="51" t="str">
+      <c r="G33" s="51" t="str">
         <f aca="false">TEXT(Inventory!D20,"#,##0")&amp;" kg · "&amp;TEXT('Nutrient balance'!D10,"0.0")&amp;" kg N"</f>
         <v>35,400 kg · 1.8 kg N</v>
       </c>
-      <c r="I60" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="J60" s="39" t="n">
+      <c r="I33" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="J33" s="39" t="n">
         <f aca="false">Inventory!D19</f>
         <v>94</v>
       </c>
-      <c r="K60" s="38" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E61" s="33" t="s">
-        <v>167</v>
-      </c>
-      <c r="I61" s="38" t="s">
-        <v>163</v>
-      </c>
-      <c r="J61" s="39" t="n">
+      <c r="K33" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E34" s="33" t="s">
+        <v>168</v>
+      </c>
+      <c r="I34" s="38" t="s">
+        <v>164</v>
+      </c>
+      <c r="J34" s="39" t="n">
         <f aca="false">Inventory!D20</f>
         <v>35400</v>
       </c>
-      <c r="K61" s="38" t="s">
+      <c r="K34" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="52" t="s">
+        <v>169</v>
+      </c>
+      <c r="B35" s="33" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="62" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="52" t="s">
-        <v>168</v>
-      </c>
-      <c r="B62" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="E62" s="53" t="s">
-        <v>169</v>
-      </c>
-      <c r="G62" s="34" t="str">
+      <c r="E35" s="53" t="s">
+        <v>170</v>
+      </c>
+      <c r="G35" s="34" t="str">
         <f aca="false">"N in products: "&amp;TEXT('Nutrient balance'!D9+'Nutrient balance'!D10,"0.0")&amp;" kg N"</f>
         <v>N in products: 6.3 kg N</v>
       </c>
-      <c r="I62" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="J62" s="44" t="n">
+      <c r="I35" s="38" t="s">
+        <v>171</v>
+      </c>
+      <c r="J35" s="44" t="n">
         <f aca="false">'Nutrient balance'!D9</f>
         <v>4.5</v>
       </c>
-      <c r="K62" s="38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="54" t="s">
+      <c r="K35" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="54" t="s">
         <v>179</v>
       </c>
-      <c r="E63" s="55" t="str">
+      <c r="E36" s="55" t="str">
         <f aca="false">IF('Nutrient balance'!D12&lt;0,"net uptake "&amp;TEXT(-'Nutrient balance'!D12,"0.0")&amp;" kg N",TEXT('Nutrient balance'!D12,"0.0")&amp;" kg N released")</f>
         <v>net uptake 0.5 kg N</v>
       </c>
-      <c r="G63" s="38" t="str">
+      <c r="G36" s="38" t="str">
         <f aca="false">"N use efficiency: "&amp;TEXT('Nutrient balance'!D13,"0%")</f>
         <v>N use efficiency: 111%</v>
       </c>
-      <c r="I63" s="38" t="s">
-        <v>172</v>
-      </c>
-      <c r="J63" s="44" t="n">
+      <c r="I36" s="38" t="s">
+        <v>173</v>
+      </c>
+      <c r="J36" s="44" t="n">
         <f aca="false">'Nutrient balance'!D10</f>
         <v>1.8</v>
       </c>
-      <c r="K63" s="38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I64" s="38" t="s">
-        <v>173</v>
-      </c>
-      <c r="J64" s="56" t="n">
+      <c r="K36" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I37" s="38" t="s">
+        <v>174</v>
+      </c>
+      <c r="J37" s="56" t="n">
         <f aca="false">'Nutrient balance'!D9+'Nutrient balance'!D10</f>
         <v>6.3</v>
       </c>
-      <c r="K64" s="38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I65" s="38" t="s">
-        <v>174</v>
-      </c>
-      <c r="J65" s="44" t="n">
+      <c r="K37" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I38" s="38" t="s">
+        <v>175</v>
+      </c>
+      <c r="J38" s="44" t="n">
         <f aca="false">'Nutrient balance'!D12</f>
         <v>-0.5</v>
       </c>
-      <c r="K65" s="38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I66" s="38" t="s">
-        <v>175</v>
-      </c>
-      <c r="J66" s="57" t="n">
+      <c r="K38" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I39" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="J39" s="57" t="n">
         <f aca="false">'Nutrient balance'!D13</f>
         <v>1.1060393258427</v>
       </c>
-      <c r="K66" s="38" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="29" t="s">
+      <c r="K39" s="38" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="59" t="s">
+    <row r="43" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="59" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="31" t="s">
-        <v>140</v>
-      </c>
-      <c r="E99" s="60" t="s">
+    <row r="45" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="F99" s="33" t="s">
+      <c r="E45" s="60" t="s">
         <v>142</v>
       </c>
-      <c r="G99" s="60" t="s">
+      <c r="F45" s="33" t="s">
         <v>143</v>
       </c>
-      <c r="I99" s="34" t="s">
+      <c r="G45" s="60" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="100" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A100" s="35" t="str">
+      <c r="I45" s="34" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="35" t="str">
         <f aca="false">TEXT(Inventory!E6,"#,##0")&amp;" kg · "&amp;TEXT('Nutrient balance'!E8,"#,##0.0")&amp;" kg N"</f>
         <v>10,975 kg · 737.5 kg N</v>
       </c>
-      <c r="B100" s="33" t="s">
-        <v>145</v>
-      </c>
-      <c r="E100" s="61" t="s">
+      <c r="B46" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="E46" s="61" t="s">
         <v>180</v>
       </c>
-      <c r="G100" s="61" t="s">
+      <c r="G46" s="61" t="s">
         <v>181</v>
       </c>
-      <c r="I100" s="37" t="s">
-        <v>147</v>
-      </c>
-      <c r="J100" s="37" t="s">
+      <c r="I46" s="37" t="s">
         <v>148</v>
       </c>
-      <c r="K100" s="37" t="s">
+      <c r="J46" s="37" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="101" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D101" s="33" t="s">
+      <c r="K46" s="37" t="s">
         <v>150</v>
       </c>
-      <c r="I101" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="J101" s="39" t="n">
+    </row>
+    <row r="47" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D47" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="I47" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="J47" s="39" t="n">
         <f aca="false">Inventory!E6</f>
         <v>10975</v>
       </c>
-      <c r="K101" s="38" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="102" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A102" s="40" t="s">
+      <c r="K47" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="40" t="s">
         <v>182</v>
       </c>
-      <c r="B102" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="C102" s="41" t="s">
+      <c r="B48" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="C48" s="41" t="s">
         <v>183</v>
       </c>
-      <c r="D102" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="E102" s="42" t="s">
-        <v>154</v>
-      </c>
-      <c r="F102" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="G102" s="43" t="s">
+      <c r="D48" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="E48" s="42" t="s">
         <v>155</v>
       </c>
-      <c r="I102" s="38" t="s">
+      <c r="F48" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="G48" s="43" t="s">
         <v>156</v>
       </c>
-      <c r="J102" s="44" t="n">
+      <c r="I48" s="38" t="s">
+        <v>157</v>
+      </c>
+      <c r="J48" s="44" t="n">
         <f aca="false">'Nutrient balance'!E8</f>
         <v>737.52</v>
       </c>
-      <c r="K102" s="38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A103" s="45" t="str">
+      <c r="K48" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="45" t="str">
         <f aca="false">TEXT(Inventory!E8+Inventory!E9,"#,##0")&amp;" kg stocked"</f>
         <v>91 kg stocked</v>
       </c>
-      <c r="C103" s="46" t="s">
-        <v>158</v>
-      </c>
-      <c r="G103" s="47" t="str">
+      <c r="C49" s="46" t="s">
+        <v>159</v>
+      </c>
+      <c r="G49" s="47" t="str">
         <f aca="false">TEXT(Inventory!E18,"#,##0")&amp;" kg gained"</f>
         <v>6,137 kg gained</v>
       </c>
-      <c r="I103" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="J103" s="39" t="n">
+      <c r="I49" s="38" t="s">
+        <v>160</v>
+      </c>
+      <c r="J49" s="39" t="n">
         <f aca="false">Inventory!E8+Inventory!E9</f>
         <v>91</v>
       </c>
-      <c r="K103" s="38" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="104" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D104" s="33" t="s">
-        <v>145</v>
-      </c>
-      <c r="I104" s="38" t="s">
-        <v>160</v>
-      </c>
-      <c r="J104" s="39" t="n">
+      <c r="K49" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D50" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="I50" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="J50" s="39" t="n">
         <f aca="false">Inventory!E7</f>
         <v>1201764</v>
       </c>
-      <c r="K104" s="38" t="s">
+      <c r="K50" s="38" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="48" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="105" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A105" s="48" t="s">
-        <v>160</v>
-      </c>
-      <c r="B105" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="E105" s="60" t="s">
-        <v>162</v>
-      </c>
-      <c r="F105" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="G105" s="60" t="s">
+      <c r="B51" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="E51" s="60" t="s">
         <v>163</v>
       </c>
-      <c r="I105" s="38" t="s">
+      <c r="F51" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="G51" s="60" t="s">
         <v>164</v>
       </c>
-      <c r="J105" s="39" t="n">
+      <c r="I51" s="38" t="s">
+        <v>165</v>
+      </c>
+      <c r="J51" s="39" t="n">
         <f aca="false">Inventory!E18</f>
         <v>6137</v>
       </c>
-      <c r="K105" s="38" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="106" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A106" s="50" t="str">
+      <c r="K51" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="50" t="str">
         <f aca="false">TEXT(Inventory!E7,"#,##0")&amp;" m3 · pumped"</f>
         <v>1,201,764 m3 · pumped</v>
       </c>
-      <c r="E106" s="61" t="s">
+      <c r="E52" s="61" t="s">
         <v>180</v>
       </c>
-      <c r="G106" s="61" t="s">
+      <c r="G52" s="61" t="s">
         <v>181</v>
       </c>
-      <c r="I106" s="38" t="s">
-        <v>166</v>
-      </c>
-      <c r="J106" s="39" t="n">
+      <c r="I52" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="J52" s="39" t="n">
         <f aca="false">Inventory!E19</f>
         <v>0</v>
       </c>
-      <c r="K106" s="38" t="s">
+      <c r="K52" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E53" s="33" t="s">
+        <v>168</v>
+      </c>
+      <c r="I53" s="38" t="s">
+        <v>164</v>
+      </c>
+      <c r="J53" s="39" t="n">
+        <f aca="false">Inventory!E20</f>
+        <v>0</v>
+      </c>
+      <c r="K53" s="38" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="52" t="s">
+        <v>169</v>
+      </c>
+      <c r="B54" s="33" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="107" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E107" s="33" t="s">
-        <v>167</v>
-      </c>
-      <c r="I107" s="38" t="s">
-        <v>163</v>
-      </c>
-      <c r="J107" s="39" t="n">
-        <f aca="false">Inventory!E20</f>
-        <v>0</v>
-      </c>
-      <c r="K107" s="38" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="108" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A108" s="52" t="s">
-        <v>168</v>
-      </c>
-      <c r="B108" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="E108" s="53" t="s">
-        <v>169</v>
-      </c>
-      <c r="G108" s="34" t="str">
+      <c r="E54" s="53" t="s">
+        <v>170</v>
+      </c>
+      <c r="G54" s="34" t="str">
         <f aca="false">"N in products: "&amp;TEXT('Nutrient balance'!E9+'Nutrient balance'!E10,"0.0")&amp;" kg N"</f>
         <v>N in products: 148.8 kg N</v>
       </c>
-      <c r="I108" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="J108" s="44" t="n">
+      <c r="I54" s="38" t="s">
+        <v>171</v>
+      </c>
+      <c r="J54" s="44" t="n">
         <f aca="false">'Nutrient balance'!E9</f>
         <v>148.8</v>
       </c>
-      <c r="K108" s="38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="109" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A109" s="54" t="s">
-        <v>171</v>
-      </c>
-      <c r="E109" s="55" t="str">
+      <c r="K54" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="54" t="s">
+        <v>172</v>
+      </c>
+      <c r="E55" s="55" t="str">
         <f aca="false">IF('Nutrient balance'!E12&lt;0,"net uptake "&amp;TEXT(-'Nutrient balance'!E12,"0.0")&amp;" kg N",TEXT('Nutrient balance'!E12,"0.0")&amp;" kg N released")</f>
         <v>588.7 kg N released</v>
       </c>
-      <c r="G109" s="38" t="str">
+      <c r="G55" s="38" t="str">
         <f aca="false">"N use efficiency: "&amp;TEXT('Nutrient balance'!E13,"0%")</f>
         <v>N use efficiency: 20%</v>
       </c>
-      <c r="I109" s="38" t="s">
-        <v>172</v>
-      </c>
-      <c r="J109" s="44" t="n">
+      <c r="I55" s="38" t="s">
+        <v>173</v>
+      </c>
+      <c r="J55" s="44" t="n">
         <f aca="false">'Nutrient balance'!E10</f>
         <v>0</v>
       </c>
-      <c r="K109" s="38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I110" s="38" t="s">
-        <v>173</v>
-      </c>
-      <c r="J110" s="56" t="n">
+      <c r="K55" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I56" s="38" t="s">
+        <v>174</v>
+      </c>
+      <c r="J56" s="56" t="n">
         <f aca="false">'Nutrient balance'!E9+'Nutrient balance'!E10</f>
         <v>148.8</v>
       </c>
-      <c r="K110" s="38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I111" s="38" t="s">
-        <v>174</v>
-      </c>
-      <c r="J111" s="44" t="n">
+      <c r="K56" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I57" s="38" t="s">
+        <v>175</v>
+      </c>
+      <c r="J57" s="44" t="n">
         <f aca="false">'Nutrient balance'!E12</f>
         <v>588.7</v>
       </c>
-      <c r="K111" s="38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I112" s="38" t="s">
-        <v>175</v>
-      </c>
-      <c r="J112" s="57" t="n">
+      <c r="K57" s="38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I58" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="J58" s="57" t="n">
         <f aca="false">'Nutrient balance'!E13</f>
         <v>0.201757240481614</v>
       </c>
-      <c r="K112" s="38" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="29" t="s">
+      <c r="K58" s="38" t="s">
         <v>177</v>
       </c>
     </row>
@@ -26328,7 +26197,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -26352,7 +26220,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26363,7 +26231,7 @@
         <v>186</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26415,7 +26283,7 @@
         <v>187</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>196</v>
@@ -26470,7 +26338,7 @@
         <v>201</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>206</v>
@@ -26478,10 +26346,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>207</v>
@@ -26489,7 +26357,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>6</v>
@@ -26541,7 +26409,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26549,7 +26417,7 @@
         <v>213</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>11</v>
@@ -26589,7 +26457,7 @@
         <v>218</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C6" s="62" t="n">
         <v>1888</v>
@@ -26609,7 +26477,7 @@
         <v>219</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C7" s="62" t="n">
         <v>101110</v>
@@ -26629,7 +26497,7 @@
         <v>220</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C8" s="62" t="n">
         <v>677</v>
@@ -26669,7 +26537,7 @@
         <v>225</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C10" s="62" t="n">
         <v>42</v>
@@ -26689,7 +26557,7 @@
         <v>226</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C11" s="62" t="n">
         <v>18</v>
@@ -26709,7 +26577,7 @@
         <v>227</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C12" s="62" t="n">
         <v>3</v>
@@ -26729,7 +26597,7 @@
         <v>228</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C13" s="62" t="n">
         <v>9</v>
@@ -26749,7 +26617,7 @@
         <v>229</v>
       </c>
       <c r="B14" s="38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C14" s="62" t="n">
         <v>1.4</v>
@@ -26829,7 +26697,7 @@
         <v>234</v>
       </c>
       <c r="B18" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C18" s="62" t="n">
         <v>1099</v>
@@ -26869,7 +26737,7 @@
         <v>236</v>
       </c>
       <c r="B20" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C20" s="62" t="n">
         <v>1224</v>
@@ -26919,7 +26787,7 @@
         <v>241</v>
       </c>
       <c r="B24" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C24" s="64" t="n">
         <f aca="false">C18+C19</f>
@@ -27061,15 +26929,15 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>11</v>
@@ -27107,10 +26975,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C8" s="67" t="n">
         <f aca="false">Inventory!C6*Inventory!C10/100/$C$5</f>
@@ -27130,10 +26998,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C9" s="68" t="n">
         <v>29</v>
@@ -27145,15 +27013,15 @@
         <v>148.8</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C10" s="68" t="n">
         <v>30.6</v>
@@ -27165,7 +27033,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27173,7 +27041,7 @@
         <v>258</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C11" s="44" t="n">
         <f aca="false">C8-C9-C10</f>
@@ -27196,7 +27064,7 @@
         <v>260</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C12" s="68" t="n">
         <v>67.2</v>
@@ -27213,10 +27081,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C13" s="69" t="n">
         <f aca="false">(C9+C10)/C8</f>
@@ -27239,7 +27107,7 @@
         <v>263</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C14" s="70" t="n">
         <f aca="false">C11*Inventory!C25</f>
@@ -27272,7 +27140,7 @@
         <v>266</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C17" s="67" t="n">
         <f aca="false">Inventory!C6*Inventory!C14/100</f>
@@ -27295,7 +27163,7 @@
         <v>267</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C18" s="68" t="n">
         <v>5.9</v>
@@ -27307,7 +27175,7 @@
         <v>25</v>
       </c>
       <c r="F18" s="29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27315,7 +27183,7 @@
         <v>268</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C19" s="68" t="n">
         <v>2.6</v>
@@ -27327,7 +27195,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27335,7 +27203,7 @@
         <v>269</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C20" s="44" t="n">
         <f aca="false">C17-C18-C19</f>
@@ -27358,7 +27226,7 @@
         <v>270</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C21" s="68" t="n">
         <v>18</v>
@@ -27378,7 +27246,7 @@
         <v>271</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C22" s="69" t="n">
         <f aca="false">(C18+C19)/C17</f>
@@ -27401,7 +27269,7 @@
         <v>272</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C23" s="70" t="n">
         <f aca="false">C20*Inventory!C25</f>
@@ -27452,7 +27320,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27488,7 +27356,7 @@
         <v>19</v>
       </c>
       <c r="F6" s="73" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G6" s="73" t="s">
         <v>278</v>
@@ -27519,7 +27387,7 @@
         <v>1788.33306175656</v>
       </c>
       <c r="F8" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G8" s="29" t="s">
         <v>282</v>
@@ -27545,7 +27413,7 @@
         <v>14.8280919015806</v>
       </c>
       <c r="F9" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G9" s="29" t="s">
         <v>284</v>
@@ -27571,7 +27439,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G10" s="29"/>
     </row>
@@ -27600,7 +27468,7 @@
         <v>195822.71468144</v>
       </c>
       <c r="F12" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G12" s="29" t="s">
         <v>289</v>
@@ -27791,7 +27659,7 @@
         <v>19</v>
       </c>
       <c r="F24" s="78" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G24" s="78" t="s">
         <v>278</v>
@@ -27848,7 +27716,7 @@
         <v>1000</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G27" s="29" t="s">
         <v>314</v>
@@ -27874,7 +27742,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G28" s="29" t="s">
         <v>314</v>
@@ -27905,7 +27773,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G30" s="29" t="s">
         <v>319</v>
@@ -27936,7 +27804,7 @@
         <v>95.9296072999837</v>
       </c>
       <c r="F32" s="38" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G32" s="29" t="s">
         <v>323</v>
@@ -28001,7 +27869,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28014,7 +27882,7 @@
         <v>328</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>11</v>
@@ -30250,7 +30118,7 @@
         <v>333</v>
       </c>
       <c r="B96" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C96" s="81" t="n">
         <v>1</v>
@@ -30279,7 +30147,7 @@
         <v>335</v>
       </c>
       <c r="B97" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C97" s="81" t="n">
         <v>38</v>
@@ -30308,7 +30176,7 @@
         <v>336</v>
       </c>
       <c r="B98" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C98" s="81" t="n">
         <v>82261</v>
@@ -30337,7 +30205,7 @@
         <v>337</v>
       </c>
       <c r="B99" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C99" s="81" t="n">
         <v>1</v>
@@ -30366,7 +30234,7 @@
         <v>338</v>
       </c>
       <c r="B100" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C100" s="81" t="n">
         <v>0</v>
@@ -30395,7 +30263,7 @@
         <v>339</v>
       </c>
       <c r="B101" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C101" s="81" t="n">
         <v>0</v>
@@ -30424,7 +30292,7 @@
         <v>340</v>
       </c>
       <c r="B102" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C102" s="81" t="n">
         <v>6</v>
@@ -30453,7 +30321,7 @@
         <v>182</v>
       </c>
       <c r="B103" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C103" s="81" t="n">
         <v>148</v>
@@ -30482,7 +30350,7 @@
         <v>341</v>
       </c>
       <c r="B104" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C104" s="81" t="n">
         <v>47</v>
@@ -30511,7 +30379,7 @@
         <v>342</v>
       </c>
       <c r="B105" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C105" s="81" t="n">
         <v>3</v>
@@ -30540,7 +30408,7 @@
         <v>343</v>
       </c>
       <c r="B106" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C106" s="81" t="n">
         <v>81336</v>
@@ -30586,7 +30454,7 @@
         <v>345</v>
       </c>
       <c r="B108" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C108" s="81" t="n">
         <v>163840</v>
@@ -30630,7 +30498,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>